<commit_message>
Actualizar proyección Chaqueta Lite con dashboards adjuntos Jacket 1.0 + 2.0
- Combina ventas DAMA de ambos dashboards
- Tolón proyectado al 85% de Chacao
- Web proyectada al 50% de Cerro Verde
- Barquisimeto como promedio Grieta + Chacao + Tolón proy.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -45,15 +45,15 @@
       <i val="1"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <i val="1"/>
+      <color rgb="00E65100"/>
     </font>
     <font>
       <b val="1"/>
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -95,6 +95,11 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -122,11 +127,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -152,11 +156,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -170,11 +172,11 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -542,11 +544,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -565,31 +567,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CUADRO JACKET 2.0 — ventas DAMA (importado, producto similar)</t>
+          <t>Jacket 1.0 + Jacket 2.0 — ventas DAMA combinadas</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fuente datos</t>
+          <t>Fuentes datos</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Dashboard_Jacket_2_0 (3).html</t>
+          <t>Dashboard_Jacket_1_0.html + Dashboard_Jacket_2_0.html</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Período referencia</t>
+          <t>Período velocidad base</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Últimos 3 meses: marzo-2026, abril-2026, mayo-2026</t>
+          <t>Jun–Jul–Ago 2026 (junio-2026, julio-2026, agosto-2026)</t>
         </is>
       </c>
     </row>
@@ -603,11 +605,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Velocidad base (3m, red actual)</t>
+          <t>Velocidad base (3m combinado)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>300</v>
+        <v>351.7</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -622,7 +624,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>269.2</v>
+        <v>321.6</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -637,7 +639,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>308</v>
+        <v>685</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -667,7 +669,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>375</v>
+        <v>439.6</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -678,15 +680,15 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Factor expansión red (Barquisimeto + Web)</t>
+          <t>Barquisimeto adicional (tienda nueva)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1.178</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>×</t>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
@@ -697,7 +699,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>441.9</v>
+        <v>503.7</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -751,7 +753,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1270</v>
+        <v>1448</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -766,7 +768,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1779</v>
+        <v>2027</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -819,7 +821,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>82.8%</t>
+          <t>81.1%</t>
         </is>
       </c>
     </row>
@@ -831,18 +833,18 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>18.9%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tope producción (cierre 60 cm)</t>
+          <t>TOPE DURO PRODUCCIÓN</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>902</v>
+        <v>921</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -853,60 +855,60 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Tope producción (cierre 75 cm)</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>4337</v>
-      </c>
-      <c r="C29" t="inlineStr">
+          <t>¿Limitado por cierres?</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SÍ</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>── RANGO DE PRODUCCIÓN SUGERIDO ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MÍNIMO (compromiso)</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>801</v>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>TOPE DURO PRODUCCIÓN</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>902</v>
-      </c>
-      <c r="C30" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MÁXIMO (techo con cierres)</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>921</v>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>und</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>¿Limitado por cierres?</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>SÍ</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>── RANGO DE PRODUCCIÓN SUGERIDO ──</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>MÍNIMO (compromiso)</t>
+          <t>Rango de acción</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>785</v>
+        <v>120</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -914,160 +916,132 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>MÁXIMO (techo con cierres)</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>902</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-    </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>Rango de acción</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>117</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>und</t>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Tolón histórico</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>── TIENDAS ──</t>
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Tolón proyectado (85% Chacao)</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>60.4</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tiendas físicas incluidas</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>SAMBIL, GRIETA, CERRO VERDE, CHACAO, GRAND PLAZ, TOLON</t>
+          <t>Web histórica</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Canal Web</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>SÍ incluido</t>
+          <t>Web proyectada (50% Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>31</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Tienda nueva BARQUISIMETO</t>
+          <t>Corporativo</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Promedio ['GRIETA', 'CHACAO', 'TOLON'] × 0.85 ramp-up</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>Velocidad mensual BARQUISIMETO (proy.)</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+          <t>EXCLUIDO</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Velocidad mensual WEB (proy.)</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>18</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
           <t>• Cierres 60 cm → XS, S, M | Cierres 75 cm → L, XL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>• La producción está limitada por cierres 60 cm (~902 und máx teórico).</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>• Barquisimeto proyectada como promedio mensual Grieta + Chacao + Tolón.</t>
         </is>
       </c>
     </row>
@@ -1095,212 +1069,212 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>CHAQUETA LITE — CANTIDADES POR TALLA (MÍN / MÁX)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>DAMA · Curva basada en Jacket 2.0 DAMA</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>DAMA · Curva Jacket 1.0 + 2.0 DAMA combinado</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Curva %</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Cierre (cm)</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>Mínimo</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Máximo</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Cierres Mín</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>Cierres Máx</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>22.4%</t>
+          <t>24.3%</t>
         </is>
       </c>
       <c r="C5" t="n">
         <v>60</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>175</v>
-      </c>
-      <c r="E5" s="9" t="n">
-        <v>202</v>
+      <c r="D5" s="7" t="n">
+        <v>194</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>223</v>
       </c>
       <c r="F5" t="n">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="G5" t="n">
-        <v>202</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>31.5%</t>
+          <t>29.2%</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>60</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>247</v>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>284</v>
+      <c r="D6" s="7" t="n">
+        <v>234</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>268</v>
       </c>
       <c r="F6" t="n">
-        <v>247</v>
+        <v>234</v>
       </c>
       <c r="G6" t="n">
-        <v>284</v>
+        <v>268</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>29.0%</t>
+          <t>27.7%</t>
         </is>
       </c>
       <c r="C7" t="n">
         <v>60</v>
       </c>
-      <c r="D7" s="8" t="n">
-        <v>228</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>262</v>
+      <c r="D7" s="7" t="n">
+        <v>222</v>
+      </c>
+      <c r="E7" s="8" t="n">
+        <v>255</v>
       </c>
       <c r="F7" t="n">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="G7" t="n">
-        <v>262</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>11.4%</t>
+          <t>15.3%</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>75</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>89</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>103</v>
+      <c r="D8" s="7" t="n">
+        <v>122</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>141</v>
       </c>
       <c r="F8" t="n">
-        <v>89</v>
+        <v>122</v>
       </c>
       <c r="G8" t="n">
-        <v>103</v>
+        <v>141</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>5.8%</t>
+          <t>3.6%</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>75</v>
       </c>
-      <c r="D9" s="8" t="n">
-        <v>46</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>51</v>
+      <c r="D9" s="7" t="n">
+        <v>29</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>34</v>
       </c>
       <c r="F9" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="G9" t="n">
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D10" s="11" t="n">
-        <v>785</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>902</v>
-      </c>
-      <c r="F10" s="11" t="n">
+      <c r="D10" s="10" t="n">
+        <v>801</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>921</v>
+      </c>
+      <c r="F10" s="10" t="n">
         <v>650</v>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>748</v>
+      <c r="G10" s="10" t="n">
+        <v>746</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Disponible cierres 60 cm</t>
         </is>
@@ -1310,12 +1284,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 748 (100%)</t>
+          <t>Usa máx 746 (100%)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>Disponible cierres 75 cm</t>
         </is>
@@ -1325,7 +1299,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Usa máx 154 (21%)</t>
+          <t>Usa máx 175 (24%)</t>
         </is>
       </c>
     </row>
@@ -1343,10 +1317,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
@@ -1360,9 +1334,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>CHAQUETA LITE — DISTRIBUCIÓN POR TIENDA Y TALLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>★ = Tolón/Web/Barquisimeto con ajuste proyectado</t>
         </is>
       </c>
     </row>
@@ -1372,527 +1353,625 @@
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>XS</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr"/>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="8" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="7" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="8" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="J4" s="8" t="inlineStr">
+      <c r="J4" s="7" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>SAMBIL</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
-        <v>43</v>
-      </c>
-      <c r="C5" s="17" t="n">
-        <v>49</v>
-      </c>
-      <c r="D5" s="16" t="n">
-        <v>60</v>
-      </c>
-      <c r="E5" s="17" t="n">
-        <v>69</v>
-      </c>
-      <c r="F5" s="16" t="n">
-        <v>56</v>
-      </c>
-      <c r="G5" s="17" t="n">
-        <v>64</v>
-      </c>
-      <c r="H5" s="16" t="n">
+      <c r="B5" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>48</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>54</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <v>51</v>
+      </c>
+      <c r="H5" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="I5" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="J5" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" s="16" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>GRIETA</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G6" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="H6" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="I6" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="J6" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>CERRO VERDE</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G7" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="J7" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>CHACAO</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>34</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>36</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>41</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>34</v>
+      </c>
+      <c r="G8" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="H8" s="15" t="n">
+        <v>19</v>
+      </c>
+      <c r="I8" s="16" t="n">
         <v>22</v>
       </c>
-      <c r="I5" s="17" t="n">
+      <c r="J8" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>GRAND PLAZ</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>LA VELA</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J10" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>TOLON ★</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="16" t="n">
-        <v>11</v>
-      </c>
-      <c r="K5" s="17" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="15" t="inlineStr">
-        <is>
-          <t>GRIETA</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="n">
+      <c r="C11" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>29</v>
+      </c>
+      <c r="G11" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="C6" s="17" t="n">
-        <v>39</v>
-      </c>
-      <c r="D6" s="16" t="n">
-        <v>48</v>
-      </c>
-      <c r="E6" s="17" t="n">
-        <v>55</v>
-      </c>
-      <c r="F6" s="16" t="n">
-        <v>44</v>
-      </c>
-      <c r="G6" s="17" t="n">
-        <v>51</v>
-      </c>
-      <c r="H6" s="16" t="n">
+      <c r="H11" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="J11" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>WEB ★</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>13</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="F12" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="G12" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="H12" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="J12" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="16" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>BARQUISIMETO ★</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="H13" s="15" t="n">
+        <v>17</v>
+      </c>
+      <c r="I13" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="J6" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="K6" s="17" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
-        <is>
-          <t>CERRO VERDE</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="C7" s="17" t="n">
-        <v>37</v>
-      </c>
-      <c r="D7" s="16" t="n">
-        <v>45</v>
-      </c>
-      <c r="E7" s="17" t="n">
-        <v>52</v>
-      </c>
-      <c r="F7" s="16" t="n">
-        <v>42</v>
-      </c>
-      <c r="G7" s="17" t="n">
-        <v>48</v>
-      </c>
-      <c r="H7" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="I7" s="17" t="n">
-        <v>19</v>
-      </c>
-      <c r="J7" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="K7" s="17" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>CHACAO</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="C8" s="17" t="n">
-        <v>37</v>
-      </c>
-      <c r="D8" s="16" t="n">
-        <v>45</v>
-      </c>
-      <c r="E8" s="17" t="n">
-        <v>52</v>
-      </c>
-      <c r="F8" s="16" t="n">
-        <v>42</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <v>48</v>
-      </c>
-      <c r="H8" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="I8" s="17" t="n">
-        <v>19</v>
-      </c>
-      <c r="J8" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="K8" s="17" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
-        <is>
-          <t>GRAND PLAZ</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="n">
+      <c r="J13" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="K13" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <v>7</v>
-      </c>
-      <c r="H9" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="I9" s="17" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="K9" s="17" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
-        <is>
-          <t>TOLON</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D10" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="E10" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="H10" s="16" t="n">
-        <v>2</v>
-      </c>
-      <c r="I10" s="17" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
-        <is>
-          <t>BARQUISIMETO ★</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="n">
-        <v>18</v>
-      </c>
-      <c r="C11" s="17" t="n">
-        <v>20</v>
-      </c>
-      <c r="D11" s="16" t="n">
-        <v>25</v>
-      </c>
-      <c r="E11" s="17" t="n">
-        <v>29</v>
-      </c>
-      <c r="F11" s="16" t="n">
-        <v>23</v>
-      </c>
-      <c r="G11" s="17" t="n">
-        <v>26</v>
-      </c>
-      <c r="H11" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="I11" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="J11" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="K11" s="17" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
-        <is>
-          <t>WEB ★</t>
-        </is>
-      </c>
-      <c r="B12" s="16" t="n">
-        <v>9</v>
-      </c>
-      <c r="C12" s="17" t="n">
-        <v>10</v>
-      </c>
-      <c r="D12" s="16" t="n">
-        <v>13</v>
-      </c>
-      <c r="E12" s="17" t="n">
-        <v>14</v>
-      </c>
-      <c r="F12" s="16" t="n">
-        <v>12</v>
-      </c>
-      <c r="G12" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="H12" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="I12" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="J12" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="17" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
-        <v>175</v>
-      </c>
-      <c r="C13" s="11" t="n">
-        <v>201</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>246</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>283</v>
-      </c>
-      <c r="F13" s="11" t="n">
-        <v>229</v>
-      </c>
-      <c r="G13" s="11" t="n">
-        <v>262</v>
-      </c>
-      <c r="H13" s="11" t="n">
-        <v>89</v>
-      </c>
-      <c r="I13" s="11" t="n">
-        <v>103</v>
-      </c>
-      <c r="J13" s="11" t="n">
-        <v>46</v>
-      </c>
-      <c r="K13" s="11" t="n">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="B14" s="10" t="n">
+        <v>194</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>223</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>234</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>268</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>222</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>255</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>123</v>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>141</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="K14" s="10" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Totales por tienda (Mín / Máx):</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>SAMBIL</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>192</v>
-      </c>
-      <c r="C16" t="n">
-        <v>219</v>
-      </c>
-    </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>GRIETA</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>152</v>
-      </c>
-      <c r="C17" t="n">
-        <v>175</v>
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Tienda</t>
+        </is>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="D17" s="19" t="inlineStr">
+        <is>
+          <t>Vel. mensual proy.</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CERRO VERDE</t>
+          <t>SAMBIL</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>144</v>
+        <v>163</v>
       </c>
       <c r="C18" t="n">
-        <v>166</v>
+        <v>185</v>
+      </c>
+      <c r="D18" t="n">
+        <v>93.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CHACAO</t>
+          <t>GRIETA</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>144</v>
+        <v>106</v>
       </c>
       <c r="C19" t="n">
-        <v>166</v>
+        <v>122</v>
+      </c>
+      <c r="D19" t="n">
+        <v>61</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GRAND PLAZ</t>
+          <t>CERRO VERDE</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>20</v>
+        <v>108</v>
       </c>
       <c r="C20" t="n">
-        <v>23</v>
+        <v>124</v>
+      </c>
+      <c r="D20" t="n">
+        <v>62.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TOLON</t>
+          <t>CHACAO</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>14</v>
+        <v>123</v>
       </c>
       <c r="C21" t="n">
-        <v>16</v>
+        <v>142</v>
+      </c>
+      <c r="D21" t="n">
+        <v>71</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BARQUISIMETO</t>
+          <t>GRAND PLAZ</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>79</v>
+        <v>14</v>
       </c>
       <c r="C22" t="n">
-        <v>91</v>
+        <v>17</v>
+      </c>
+      <c r="D22" t="n">
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>LA VELA</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="C23" t="n">
-        <v>46</v>
+        <v>20</v>
+      </c>
+      <c r="D23" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TOLON ★</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>105</v>
+      </c>
+      <c r="C24" t="n">
+        <v>121</v>
+      </c>
+      <c r="D24" t="n">
+        <v>60.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>WEB ★</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>54</v>
+      </c>
+      <c r="C25" t="n">
+        <v>62</v>
+      </c>
+      <c r="D25" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BARQUISIMETO ★</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>111</v>
+      </c>
+      <c r="C26" t="n">
+        <v>128</v>
+      </c>
+      <c r="D26" t="n">
+        <v>64.09999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1914,17 +1993,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1934,325 +2006,133 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>QX Negro 0580</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Modelo</t>
+          <t>Color producto</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>QX Negro 0580</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Color producto</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
           <t>Negro (inferido del insumo)</t>
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
+        <is>
+          <t>Longitud</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Tallas</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="inlineStr">
+        <is>
+          <t>Disponible</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="inlineStr">
+        <is>
+          <t>Usa Mín</t>
+        </is>
+      </c>
+      <c r="E5" s="21" t="inlineStr">
+        <is>
+          <t>Usa Máx</t>
+        </is>
+      </c>
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>Remanente Mín</t>
+        </is>
+      </c>
+      <c r="G5" s="21" t="inlineStr">
+        <is>
+          <t>Remanente Máx</t>
+        </is>
+      </c>
+      <c r="H5" s="21" t="inlineStr">
+        <is>
+          <t>% uso máx</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>Longitud</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Tallas</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>Disponible</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>Usa Mín</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>Usa Máx</t>
-        </is>
-      </c>
-      <c r="F6" s="21" t="inlineStr">
-        <is>
-          <t>Remanente Mín</t>
-        </is>
-      </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>Remanente Máx</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>% uso máx</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>60 cm</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>XS · S · M</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>748</v>
+      </c>
+      <c r="D6" t="n">
+        <v>650</v>
+      </c>
+      <c r="E6" t="n">
+        <v>746</v>
+      </c>
+      <c r="F6" t="n">
+        <v>98</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>100%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>60 cm</t>
+          <t>75 cm</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>XS · S · M</t>
+          <t>L · XL</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>748</v>
+        <v>744</v>
       </c>
       <c r="D7" t="n">
-        <v>650</v>
+        <v>151</v>
       </c>
       <c r="E7" t="n">
-        <v>748</v>
+        <v>175</v>
       </c>
       <c r="F7" t="n">
-        <v>98</v>
+        <v>593</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>569</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>100%</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>75 cm</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>L · XL</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>744</v>
-      </c>
-      <c r="D8" t="n">
-        <v>135</v>
-      </c>
-      <c r="E8" t="n">
-        <v>154</v>
-      </c>
-      <c r="F8" t="n">
-        <v>609</v>
-      </c>
-      <c r="G8" t="n">
-        <v>590</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>21%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Detalle por talla (Mín / Máx)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Talla</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Cierre</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>XS</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>60 cm</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>175</v>
-      </c>
-      <c r="D12" t="n">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="B13" s="22" t="inlineStr">
-        <is>
-          <t>60 cm</t>
-        </is>
-      </c>
-      <c r="C13" s="22" t="n">
-        <v>247</v>
-      </c>
-      <c r="D13" s="22" t="n">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>60 cm</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>228</v>
-      </c>
-      <c r="D14" t="n">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>75 cm</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>89</v>
-      </c>
-      <c r="D15" t="n">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>75 cm</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>46</v>
-      </c>
-      <c r="D16" t="n">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Tope teórico si se agotan todos los cierres 60 cm</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>902</v>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Cierres 75 cm necesarios al tope</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>155</v>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Cierres 75 cm sobrantes al tope</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>589</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Recomendación</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>• El cierre 60 cm es el INSUMO LIMITANTE — planificar producción desde este tope.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>• Al máximo de producción se usan ~100% cierres 60 cm y ~21% cierres 75 cm.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>• Reservar remanente 75 cm para reposición o segunda producción.</t>
+          <t>24%</t>
         </is>
       </c>
     </row>
@@ -2267,14 +2147,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>METODOLOGÍA — PROYECCIÓN CHAQUETA LITE</t>
         </is>
@@ -2284,7 +2164,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>1. PRODUCTO DE REFERENCIA</t>
         </is>
@@ -2293,21 +2173,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Se usó CUADRO JACKET 2.0 (importado) filtrado a género DAMA como proxy de demanda.</t>
+          <t xml:space="preserve">   Fuentes: Dashboard_Jacket_1_0.html + Dashboard_Jacket_2_0.html (adjuntos).</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Jacket 1.0 no estaba disponible en el repositorio; Jacket 2.0 tiene 6 meses de historial.</t>
+          <t xml:space="preserve">   Se combinaron ventas DAMA de Jacket 1.0 y CUADRO Jacket 2.0.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Velocidad base = promedio últimos 3 meses (Mar–May 2026): 300 und/mes.</t>
+          <t xml:space="preserve">   Velocidad base = promedio Jun–Jul–Ago 2026: 352 und/mes.</t>
         </is>
       </c>
     </row>
@@ -2315,7 +2195,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>2. AJUSTE TEMPORADA ALTA</t>
         </is>
@@ -2324,186 +2204,148 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Factor ×1.25 aplicado (diciembre + regalos navideños).</t>
+          <t xml:space="preserve">   Factor ×1.25 (diciembre). Diciembre 2025 combinado: 685 und.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Diciembre 2025 Jacket DAMA vendió 308 und (1.03× vs base 3m).</t>
-        </is>
-      </c>
+      <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>3. AJUSTES DE TIENDA (según indicación)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>3. EXPANSIÓN DE RED</t>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Tolón: proyectado al 85% de Chacao (71 → 60 und/mes).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Barquisimeto (nueva): promedio mensual Grieta + Chacao + Tolón × ramp-up 0.85.</t>
+          <t xml:space="preserve">     Histórico Tolón: 8 und/mes — subestimado por tienda nueva.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">     → 36 und/mes proyectadas.</t>
+          <t xml:space="preserve">   • Web: proyectada al 50% de Cerro Verde (62 → 31 und/mes).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Web: 6% de velocidad base → 18 und/mes.</t>
+          <t xml:space="preserve">     Histórico Web: 8 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t xml:space="preserve">   • Barquisimeto (nueva): promedio Grieta + Chacao + Tolón proyectado = 64 und/mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t xml:space="preserve">   • Corporativo: EXCLUIDO.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>4. COBERTURA Y STOCK DE SEGURIDAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Mínimo: 2.5 meses de venta a velocidad ajustada + 15% SS.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Máximo: 3.5 meses o mín × 1.12, lo que aplique.</t>
+          <t xml:space="preserve">   Mínimo: 2.5 meses + 15% SS.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Máximo: 3.5 meses o mín × 1.12.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>5. INSUMO LIMITANTE — CIERRES</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   QX Negro 0580: 60 cm (748 und) para XS/S/M | 75 cm (744 und) para L/XL.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Curva tallas Jacket DAMA: 60 cm = 82.8%, 75 cm = 17.2%.</t>
+          <t xml:space="preserve">   Tope duro = 921 und (cierre 60 cm limitante).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Tope duro = 902 und (limitado por cierres 60 cm).</t>
-        </is>
-      </c>
+      <c r="A25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" s="19" t="inlineStr">
+        <is>
+          <t>6. RANGO MÍNIMO / MÁXIMO</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>6. RANGO MÍNIMO / MÁXIMO</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Demanda teórica mín: 1448 → ajustada: 801 und.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Demanda teórica mín: 1270 und → ajustada a 785 und (cap cierres).</t>
+          <t xml:space="preserve">   Demanda teórica máx: 2027 → ajustada: 921 und.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Demanda teórica máx: 1779 und → ajustada a 902 und (cap cierres).</t>
-        </is>
-      </c>
+      <c r="A29" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr"/>
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>7. DISTRIBUCIÓN</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>7. DISTRIBUCIÓN</t>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Por tienda: participación histórica Jacket DAMA + Barquisimeto + Web.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por talla: curva histórica Jacket DAMA (XS 22%, S 32%, M 29%, L 11%, XL 6%).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>8. DECISIÓN EN REUNIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • MÍNIMO = compromiso de producción para cubrir temporada alta + SS dentro del cap de cierres.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • MÁXIMO = techo si se confirma demanda fuerte; no supera cierres 60 cm disponibles.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Distribuir a tiendas y mover entre puntos de venta según rotación real post-lanzamiento.</t>
+          <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajustar La Vela (avg Sambil+Cerro Verde) y Grand Plaz (+20%) en proyección Chaqueta Lite
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -169,11 +169,11 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -986,11 +986,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>64.09999999999999</v>
+        <v>10</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1001,45 +1001,105 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Grand Plaz histórica</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Grand Plaz proyectada (+20%)</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>10</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>• Cierres 60 cm → XS, S, M | Cierres 75 cm → L, XL.</t>
         </is>
@@ -1343,7 +1403,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>★ = Tolón/Web/Barquisimeto con ajuste proyectado</t>
+          <t>★ = tienda con velocidad proyectada/ajustada</t>
         </is>
       </c>
     </row>
@@ -1438,34 +1498,34 @@
         </is>
       </c>
       <c r="B5" s="15" t="n">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C5" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="D5" s="15" t="n">
+        <v>41</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>47</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>39</v>
+      </c>
+      <c r="G5" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="D5" s="15" t="n">
-        <v>48</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>54</v>
-      </c>
-      <c r="F5" s="15" t="n">
-        <v>45</v>
-      </c>
-      <c r="G5" s="16" t="n">
-        <v>51</v>
-      </c>
       <c r="H5" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="I5" s="16" t="n">
         <v>25</v>
-      </c>
-      <c r="I5" s="16" t="n">
-        <v>28</v>
       </c>
       <c r="J5" s="15" t="n">
         <v>5</v>
       </c>
       <c r="K5" s="16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -1475,34 +1535,34 @@
         </is>
       </c>
       <c r="B6" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="C6" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="C6" s="16" t="n">
-        <v>30</v>
-      </c>
       <c r="D6" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E6" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="E6" s="16" t="n">
-        <v>36</v>
-      </c>
       <c r="F6" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="G6" s="16" t="n">
         <v>29</v>
       </c>
-      <c r="G6" s="16" t="n">
-        <v>34</v>
-      </c>
       <c r="H6" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="I6" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="I6" s="16" t="n">
-        <v>19</v>
-      </c>
       <c r="J6" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="16" t="n">
         <v>4</v>
-      </c>
-      <c r="K6" s="16" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -1512,34 +1572,34 @@
         </is>
       </c>
       <c r="B7" s="15" t="n">
+        <v>23</v>
+      </c>
+      <c r="C7" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="D7" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="G7" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="D7" s="15" t="n">
-        <v>31</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>36</v>
-      </c>
-      <c r="F7" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="G7" s="16" t="n">
-        <v>34</v>
-      </c>
       <c r="H7" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="I7" s="16" t="n">
         <v>17</v>
-      </c>
-      <c r="I7" s="16" t="n">
-        <v>19</v>
       </c>
       <c r="J7" s="15" t="n">
         <v>4</v>
       </c>
       <c r="K7" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1549,44 +1609,44 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
+        <v>26</v>
+      </c>
+      <c r="C8" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="D8" s="15" t="n">
+        <v>31</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="D8" s="15" t="n">
-        <v>36</v>
-      </c>
-      <c r="E8" s="16" t="n">
-        <v>41</v>
-      </c>
-      <c r="F8" s="15" t="n">
-        <v>34</v>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>39</v>
-      </c>
       <c r="H8" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="I8" s="16" t="n">
         <v>19</v>
-      </c>
-      <c r="I8" s="16" t="n">
-        <v>22</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="16" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
-        <is>
-          <t>GRAND PLAZ</t>
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>GRAND PLAZ ★</t>
         </is>
       </c>
       <c r="B9" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" s="16" t="n">
         <v>4</v>
@@ -1612,156 +1672,156 @@
       <c r="J9" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="K9" s="18" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>LA VELA</t>
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>LA VELA ★</t>
         </is>
       </c>
       <c r="B10" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>34</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>39</v>
+      </c>
+      <c r="F10" s="15" t="n">
+        <v>32</v>
+      </c>
+      <c r="G10" s="16" t="n">
+        <v>37</v>
+      </c>
+      <c r="H10" s="15" t="n">
+        <v>18</v>
+      </c>
+      <c r="I10" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="J10" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>TOLON ★</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
+        <v>22</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="F11" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="I11" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="J11" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="C10" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="F10" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="H10" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="I10" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="J10" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>TOLON ★</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>25</v>
-      </c>
-      <c r="C11" s="16" t="n">
-        <v>29</v>
-      </c>
-      <c r="D11" s="15" t="n">
-        <v>31</v>
-      </c>
-      <c r="E11" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="F11" s="15" t="n">
-        <v>29</v>
-      </c>
-      <c r="G11" s="16" t="n">
-        <v>34</v>
-      </c>
-      <c r="H11" s="15" t="n">
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>WEB ★</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>14</v>
+      </c>
+      <c r="E12" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="I11" s="16" t="n">
-        <v>18</v>
-      </c>
-      <c r="J11" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="K11" s="16" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t>WEB ★</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="n">
+      <c r="F12" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="G12" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="D12" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="E12" s="16" t="n">
-        <v>18</v>
-      </c>
-      <c r="F12" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="G12" s="16" t="n">
-        <v>17</v>
-      </c>
       <c r="H12" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="I12" s="16" t="n">
         <v>8</v>
-      </c>
-      <c r="I12" s="16" t="n">
-        <v>9</v>
       </c>
       <c r="J12" s="15" t="n">
         <v>2</v>
       </c>
       <c r="K12" s="16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>BARQUISIMETO ★</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>24</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>32</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>27</v>
+      </c>
+      <c r="G13" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="H13" s="15" t="n">
+        <v>15</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="J13" s="15" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="18" t="inlineStr">
-        <is>
-          <t>BARQUISIMETO ★</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n">
-        <v>27</v>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>31</v>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>37</v>
-      </c>
-      <c r="F13" s="15" t="n">
-        <v>31</v>
-      </c>
-      <c r="G13" s="16" t="n">
-        <v>35</v>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>17</v>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="J13" s="15" t="n">
+      <c r="K13" s="16" t="n">
         <v>4</v>
-      </c>
-      <c r="K13" s="16" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -1777,7 +1837,7 @@
         <v>223</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>268</v>
@@ -1789,16 +1849,16 @@
         <v>255</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16">
@@ -1837,10 +1897,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>163</v>
+        <v>141</v>
       </c>
       <c r="C18" t="n">
-        <v>185</v>
+        <v>162</v>
       </c>
       <c r="D18" t="n">
         <v>93.3</v>
@@ -1853,10 +1913,10 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>92</v>
+      </c>
+      <c r="C19" t="n">
         <v>106</v>
-      </c>
-      <c r="C19" t="n">
-        <v>122</v>
       </c>
       <c r="D19" t="n">
         <v>61</v>
@@ -1869,10 +1929,10 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>94</v>
+      </c>
+      <c r="C20" t="n">
         <v>108</v>
-      </c>
-      <c r="C20" t="n">
-        <v>124</v>
       </c>
       <c r="D20" t="n">
         <v>62.1</v>
@@ -1885,10 +1945,10 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>107</v>
+      </c>
+      <c r="C21" t="n">
         <v>123</v>
-      </c>
-      <c r="C21" t="n">
-        <v>142</v>
       </c>
       <c r="D21" t="n">
         <v>71</v>
@@ -1897,33 +1957,33 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GRAND PLAZ</t>
+          <t>GRAND PLAZ ★</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C22" t="n">
         <v>17</v>
       </c>
       <c r="D22" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LA VELA</t>
+          <t>LA VELA ★</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="C23" t="n">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>77.7</v>
       </c>
     </row>
     <row r="24">
@@ -1933,10 +1993,10 @@
         </is>
       </c>
       <c r="B24" t="n">
+        <v>91</v>
+      </c>
+      <c r="C24" t="n">
         <v>105</v>
-      </c>
-      <c r="C24" t="n">
-        <v>121</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -1949,10 +2009,10 @@
         </is>
       </c>
       <c r="B25" t="n">
+        <v>47</v>
+      </c>
+      <c r="C25" t="n">
         <v>54</v>
-      </c>
-      <c r="C25" t="n">
-        <v>62</v>
       </c>
       <c r="D25" t="n">
         <v>31</v>
@@ -1965,10 +2025,10 @@
         </is>
       </c>
       <c r="B26" t="n">
+        <v>97</v>
+      </c>
+      <c r="C26" t="n">
         <v>111</v>
-      </c>
-      <c r="C26" t="n">
-        <v>128</v>
       </c>
       <c r="D26" t="n">
         <v>64.09999999999999</v>
@@ -2147,7 +2207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -2249,38 +2309,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Barquisimeto (nueva): promedio Grieta + Chacao + Tolón proyectado = 64 und/mes.</t>
+          <t xml:space="preserve">   • La Vela (nueva): promedio Sambil + Cerro Verde = 78 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Corporativo: EXCLUIDO.</t>
+          <t xml:space="preserve">     Histórico La Vela: 10 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Grand Plaz: histórico × 1.2 = 10 und/mes.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>4. COBERTURA Y STOCK DE SEGURIDAD</t>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Histórico Grand Plaz: 8 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mínimo: 2.5 meses + 15% SS.</t>
+          <t xml:space="preserve">   • Barquisimeto (nueva): promedio Grieta + Chacao + Tolón proyectado = 64 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Máximo: 3.5 meses o mín × 1.12.</t>
+          <t xml:space="preserve">   • Corporativo: EXCLUIDO.</t>
         </is>
       </c>
     </row>
@@ -2290,38 +2354,38 @@
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>5. INSUMO LIMITANTE — CIERRES</t>
+          <t>4. COBERTURA Y STOCK DE SEGURIDAD</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Tope duro = 921 und (cierre 60 cm limitante).</t>
+          <t xml:space="preserve">   Mínimo: 2.5 meses + 15% SS.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Máximo: 3.5 meses o mín × 1.12.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="19" t="inlineStr">
-        <is>
-          <t>6. RANGO MÍNIMO / MÁXIMO</t>
-        </is>
-      </c>
+      <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Demanda teórica mín: 1448 → ajustada: 801 und.</t>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>5. INSUMO LIMITANTE — CIERRES</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Demanda teórica máx: 2027 → ajustada: 921 und.</t>
+          <t xml:space="preserve">   Tope duro = 921 und (cierre 60 cm limitante).</t>
         </is>
       </c>
     </row>
@@ -2331,19 +2395,43 @@
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>7. DISTRIBUCIÓN</t>
+          <t>6. RANGO MÍNIMO / MÁXIMO</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+          <t xml:space="preserve">   Demanda teórica mín: 1448 → ajustada: 801 und.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Demanda teórica máx: 2027 → ajustada: 921 und.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="19" t="inlineStr">
+        <is>
+          <t>7. DISTRIBUCIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
         </is>

</xml_diff>

<commit_message>
Fijar rango global 850-940 und y subir Grand Plaz a +40% histórico
- Rango de producción acordado: 850 mín / 940 máx
- Grand Plaz: +40% sobre histórico (11.7 und/mes proy.)
- Documentar déficit ~15 cierres 60 cm al producir 940 und

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -53,7 +53,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00A8C8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFCDD2"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -153,6 +158,9 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -160,7 +168,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -169,10 +177,10 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -544,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -840,7 +848,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TOPE DURO PRODUCCIÓN</t>
+          <t>Tope teórico cierres 60 cm</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -855,19 +863,19 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>¿Limitado por cierres?</t>
+          <t>¿Máximo supera cierres 60 cm?</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SÍ</t>
+          <t>SÍ — ver hoja Cierres</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>── RANGO DE PRODUCCIÓN SUGERIDO ──</t>
+          <t>── RANGO DE PRODUCCIÓN (ACORDADO) ──</t>
         </is>
       </c>
     </row>
@@ -878,7 +886,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>801</v>
+        <v>850</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -889,11 +897,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MÁXIMO (techo con cierres)</t>
+          <t>MÁXIMO</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>921</v>
+        <v>940</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -908,7 +916,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -916,51 +924,51 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Cierres 60 cm al máximo</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>763</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>de 748 disp.</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Déficit cierres 60 cm al máximo</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>15</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Tolón proyectado (85% Chacao)</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Web histórica</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -971,11 +979,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Web proyectada (50% Cerro Verde)</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>31</v>
+        <v>60.4</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -986,11 +994,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>10</v>
+        <v>7.8</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1001,11 +1009,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+          <t>Web proyectada (50% Cerro Verde)</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>77.7</v>
+        <v>31</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1016,11 +1024,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1031,11 +1039,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+20%)</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>10</v>
+        <v>77.7</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1046,11 +1054,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Grand Plaz histórica</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>64.09999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1061,45 +1069,75 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>Grand Plaz proyectada (+40% hist.)</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>• Cierres 60 cm → XS, S, M | Cierres 75 cm → L, XL.</t>
         </is>
@@ -1194,16 +1232,16 @@
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="F5" t="n">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="G5" t="n">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6">
@@ -1221,16 +1259,16 @@
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="F6" t="n">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="G6" t="n">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="7">
@@ -1248,16 +1286,16 @@
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="F7" t="n">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="G7" t="n">
-        <v>255</v>
+        <v>261</v>
       </c>
     </row>
     <row r="8">
@@ -1275,16 +1313,16 @@
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F8" t="n">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="G8" t="n">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9">
@@ -1302,16 +1340,16 @@
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F9" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G9" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10">
@@ -1321,16 +1359,16 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>801</v>
+        <v>850</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>921</v>
+        <v>940</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>650</v>
+        <v>690</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>746</v>
+        <v>763</v>
       </c>
     </row>
     <row r="12">
@@ -1344,12 +1382,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 746 (100%)</t>
+          <t>Usa máx 763 (faltan 15)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Disponible cierres 75 cm</t>
         </is>
@@ -1359,7 +1397,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Usa máx 175 (24%)</t>
+          <t>Usa máx 177 (24%)</t>
         </is>
       </c>
     </row>
@@ -1401,14 +1439,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="13" t="inlineStr">
         <is>
           <t>★ = tienda con velocidad proyectada/ajustada</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="14" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
@@ -1492,336 +1530,336 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>SAMBIL</t>
         </is>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="C5" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>44</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>48</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <v>42</v>
+      </c>
+      <c r="G5" s="17" t="n">
+        <v>45</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="J5" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" s="17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>GRIETA</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="F6" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="J6" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>CERRO VERDE</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="C7" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>32</v>
+      </c>
+      <c r="F7" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="H7" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="J7" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="K7" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>CHACAO</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="C8" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>33</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>36</v>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="J8" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="inlineStr">
+        <is>
+          <t>GRAND PLAZ ★</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="inlineStr">
+        <is>
+          <t>LA VELA ★</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="F10" s="16" t="n">
         <v>34</v>
       </c>
-      <c r="C5" s="16" t="n">
-        <v>39</v>
-      </c>
-      <c r="D5" s="15" t="n">
-        <v>41</v>
-      </c>
-      <c r="E5" s="16" t="n">
-        <v>47</v>
-      </c>
-      <c r="F5" s="15" t="n">
-        <v>39</v>
-      </c>
-      <c r="G5" s="16" t="n">
-        <v>45</v>
-      </c>
-      <c r="H5" s="15" t="n">
-        <v>22</v>
-      </c>
-      <c r="I5" s="16" t="n">
+      <c r="G10" s="17" t="n">
+        <v>38</v>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="J10" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="18" t="inlineStr">
+        <is>
+          <t>TOLON ★</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>26</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="H11" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="J11" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="18" t="inlineStr">
+        <is>
+          <t>WEB ★</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="J12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="inlineStr">
+        <is>
+          <t>BARQUISIMETO ★</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="C13" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>31</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="I13" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="J13" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="17" t="n">
         <v>5</v>
-      </c>
-      <c r="K5" s="16" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
-        <is>
-          <t>GRIETA</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="n">
-        <v>22</v>
-      </c>
-      <c r="C6" s="16" t="n">
-        <v>26</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>27</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>31</v>
-      </c>
-      <c r="F6" s="15" t="n">
-        <v>26</v>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>29</v>
-      </c>
-      <c r="H6" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="I6" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="J6" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" s="16" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="14" t="inlineStr">
-        <is>
-          <t>CERRO VERDE</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="n">
-        <v>23</v>
-      </c>
-      <c r="C7" s="16" t="n">
-        <v>26</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>27</v>
-      </c>
-      <c r="E7" s="16" t="n">
-        <v>31</v>
-      </c>
-      <c r="F7" s="15" t="n">
-        <v>26</v>
-      </c>
-      <c r="G7" s="16" t="n">
-        <v>30</v>
-      </c>
-      <c r="H7" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="I7" s="16" t="n">
-        <v>17</v>
-      </c>
-      <c r="J7" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="16" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
-        <is>
-          <t>CHACAO</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="n">
-        <v>26</v>
-      </c>
-      <c r="C8" s="16" t="n">
-        <v>30</v>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>31</v>
-      </c>
-      <c r="E8" s="16" t="n">
-        <v>36</v>
-      </c>
-      <c r="F8" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>34</v>
-      </c>
-      <c r="H8" s="15" t="n">
-        <v>16</v>
-      </c>
-      <c r="I8" s="16" t="n">
-        <v>19</v>
-      </c>
-      <c r="J8" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="16" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>GRAND PLAZ ★</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="C9" s="16" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="G9" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="I9" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>LA VELA ★</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="n">
-        <v>28</v>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>33</v>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>34</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>39</v>
-      </c>
-      <c r="F10" s="15" t="n">
-        <v>32</v>
-      </c>
-      <c r="G10" s="16" t="n">
-        <v>37</v>
-      </c>
-      <c r="H10" s="15" t="n">
-        <v>18</v>
-      </c>
-      <c r="I10" s="16" t="n">
-        <v>21</v>
-      </c>
-      <c r="J10" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="K10" s="16" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>TOLON ★</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="n">
-        <v>22</v>
-      </c>
-      <c r="C11" s="16" t="n">
-        <v>25</v>
-      </c>
-      <c r="D11" s="15" t="n">
-        <v>27</v>
-      </c>
-      <c r="E11" s="16" t="n">
-        <v>31</v>
-      </c>
-      <c r="F11" s="15" t="n">
-        <v>25</v>
-      </c>
-      <c r="G11" s="16" t="n">
-        <v>29</v>
-      </c>
-      <c r="H11" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="I11" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="J11" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="K11" s="16" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>WEB ★</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="C12" s="16" t="n">
-        <v>13</v>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>14</v>
-      </c>
-      <c r="E12" s="16" t="n">
-        <v>16</v>
-      </c>
-      <c r="F12" s="15" t="n">
-        <v>13</v>
-      </c>
-      <c r="G12" s="16" t="n">
-        <v>15</v>
-      </c>
-      <c r="H12" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="I12" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="J12" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="16" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>BARQUISIMETO ★</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n">
-        <v>24</v>
-      </c>
-      <c r="C13" s="16" t="n">
-        <v>27</v>
-      </c>
-      <c r="D13" s="15" t="n">
-        <v>28</v>
-      </c>
-      <c r="E13" s="16" t="n">
-        <v>32</v>
-      </c>
-      <c r="F13" s="15" t="n">
-        <v>27</v>
-      </c>
-      <c r="G13" s="16" t="n">
-        <v>31</v>
-      </c>
-      <c r="H13" s="15" t="n">
-        <v>15</v>
-      </c>
-      <c r="I13" s="16" t="n">
-        <v>17</v>
-      </c>
-      <c r="J13" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="16" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1831,60 +1869,60 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>233</v>
+        <v>249</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>Totales por tienda (Mín / Máx):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="D17" s="20" t="inlineStr">
         <is>
           <t>Vel. mensual proy.</t>
         </is>
@@ -1897,10 +1935,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="C18" t="n">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D18" t="n">
         <v>93.3</v>
@@ -1913,10 +1951,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C19" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D19" t="n">
         <v>61</v>
@@ -1929,10 +1967,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C20" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D20" t="n">
         <v>62.1</v>
@@ -1945,10 +1983,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C21" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D21" t="n">
         <v>71</v>
@@ -1961,13 +1999,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C22" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>11.7</v>
       </c>
     </row>
     <row r="23">
@@ -1977,10 +2015,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C23" t="n">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D23" t="n">
         <v>77.7</v>
@@ -1993,10 +2031,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C24" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -2009,10 +2047,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C25" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D25" t="n">
         <v>31</v>
@@ -2025,10 +2063,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C26" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D26" t="n">
         <v>64.09999999999999</v>
@@ -2060,7 +2098,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>PLAN DE CIERRES — QX NEGRO 0580</t>
         </is>
@@ -2091,42 +2129,42 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Longitud</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Tallas</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Usa Mín</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Usa Máx</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>Remanente Mín</t>
         </is>
       </c>
-      <c r="G5" s="21" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>Remanente Máx</t>
         </is>
       </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>% uso máx</t>
         </is>
@@ -2147,20 +2185,20 @@
         <v>748</v>
       </c>
       <c r="D6" t="n">
-        <v>650</v>
+        <v>690</v>
       </c>
       <c r="E6" t="n">
-        <v>746</v>
+        <v>763</v>
       </c>
       <c r="F6" t="n">
-        <v>98</v>
+        <v>58</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>-15</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>102%</t>
         </is>
       </c>
     </row>
@@ -2179,16 +2217,16 @@
         <v>744</v>
       </c>
       <c r="D7" t="n">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="E7" t="n">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F7" t="n">
-        <v>593</v>
+        <v>584</v>
       </c>
       <c r="G7" t="n">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -2207,14 +2245,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A36"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>METODOLOGÍA — PROYECCIÓN CHAQUETA LITE</t>
         </is>
@@ -2224,7 +2262,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>1. PRODUCTO DE REFERENCIA</t>
         </is>
@@ -2255,7 +2293,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>2. AJUSTE TEMPORADA ALTA</t>
         </is>
@@ -2272,7 +2310,7 @@
       <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>3. AJUSTES DE TIENDA (según indicación)</t>
         </is>
@@ -2323,7 +2361,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Grand Plaz: histórico × 1.2 = 10 und/mes.</t>
+          <t xml:space="preserve">   • Grand Plaz: histórico × 1.4 (+40%) = 12 und/mes.</t>
         </is>
       </c>
     </row>
@@ -2352,23 +2390,23 @@
       <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
-        <is>
-          <t>4. COBERTURA Y STOCK DE SEGURIDAD</t>
+      <c r="A23" s="20" t="inlineStr">
+        <is>
+          <t>4. RANGO GLOBAL ACORDADO</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mínimo: 2.5 meses + 15% SS.</t>
+          <t xml:space="preserve">   Mínimo: 850 und | Máximo: 940 und.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Máximo: 3.5 meses o mín × 1.12.</t>
+          <t xml:space="preserve">   Demanda teórica calculada: 1448 – 2027 und (referencia).</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2414,7 @@
       <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="20" t="inlineStr">
         <is>
           <t>5. INSUMO LIMITANTE — CIERRES</t>
         </is>
@@ -2385,53 +2423,67 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Tope duro = 921 und (cierre 60 cm limitante).</t>
+          <t xml:space="preserve">   Tope teórico cierres 60 cm = 921 und.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Al máximo (940 und) se necesitan 763 cierres 60 cm.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="19" t="inlineStr">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Déficit al máximo: 15 und de cierre 60 cm (si no se compran más).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
         <is>
           <t>6. RANGO MÍNIMO / MÁXIMO</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Demanda teórica mín: 1448 → ajustada: 801 und.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Demanda teórica máx: 2027 → ajustada: 921 und.</t>
-        </is>
-      </c>
-    </row>
     <row r="33">
-      <c r="A33" t="inlineStr"/>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Compromiso mín: 850 und.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="19" t="inlineStr">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Techo máx: 940 und.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="20" t="inlineStr">
         <is>
           <t>7. DISTRIBUCIÓN</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
         </is>

</xml_diff>

<commit_message>
Tratar cierres como inventario global intercambiable (75 cm adaptable a 60 cm)
- Pool total: 748 + 744 = 1.492 und
- Rango 850-940 cabe cómodamente con 552 und remanentes al máximo
- Asignación: 15 cierres 75 cm se adaptan para cubrir XS/S/M

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -53,7 +53,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -88,11 +88,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00A8C8E8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFCDD2"/>
       </patternFill>
     </fill>
     <fill>
@@ -132,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,9 +153,6 @@
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -168,7 +160,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -177,15 +169,14 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -552,7 +543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -794,11 +785,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cierre 60 cm (XS · S · M)</t>
+          <t>Inventario global (60 + 75 cm)</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>748</v>
+        <v>1492</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -809,50 +800,54 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cierre 75 cm (L · XL)</t>
+          <t xml:space="preserve">  · Cierres 60 cm en stock</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>und disponibles</t>
+          <t>und</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Curva tallas → % cierre 60 cm</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>81.1%</t>
+          <t xml:space="preserve">  · Cierres 75 cm en stock</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>744</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>und (adaptables a 60 cm)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Curva tallas → % cierre 75 cm</t>
+          <t>Lógica</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>18.9%</t>
-        </is>
-      </c>
+          <t>1 cierre = 1 chaqueta · pool global intercambiable</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tope teórico cierres 60 cm</t>
+          <t>Tope producción (inventario global)</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>921</v>
+        <v>1492</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -863,12 +858,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>¿Máximo supera cierres 60 cm?</t>
+          <t>¿Rango 850–940 cabe en stock?</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SÍ — ver hoja Cierres</t>
+          <t>SÍ</t>
         </is>
       </c>
     </row>
@@ -927,63 +922,63 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cierres 60 cm al máximo</t>
+          <t>Cierres usados al mínimo</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>763</v>
+        <v>850</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>de 748 disp.</t>
+          <t>de 1492 disp.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Déficit cierres 60 cm al máximo</t>
+          <t>Cierres usados al máximo</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>15</v>
+        <v>940</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
+          <t>de 1492 disp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Remanente global al máximo</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>552</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
           <t>und</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>60.4</v>
+        <v>8.1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -994,11 +989,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Web histórica</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>7.8</v>
+        <v>60.4</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1009,11 +1004,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Web proyectada (50% Cerro Verde)</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>31</v>
+        <v>7.8</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1024,11 +1019,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
+          <t>Web proyectada (50% Cerro Verde)</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1039,11 +1034,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>77.7</v>
+        <v>10</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1054,11 +1049,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>8.300000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1069,11 +1064,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+40% hist.)</t>
+          <t>Grand Plaz histórica</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>11.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1084,11 +1079,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Grand Plaz proyectada (+40% hist.)</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>64.09999999999999</v>
+        <v>11.7</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1099,47 +1094,62 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>Corporativo</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>EXCLUIDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>• Cierres 60 cm → XS, S, M | Cierres 75 cm → L, XL.</t>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
       </c>
     </row>
@@ -1374,30 +1384,30 @@
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>Disponible cierres 60 cm</t>
+          <t>Inventario global cierres</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>748</v>
+        <v>1492</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 763 (faltan 15)</t>
+          <t>Usa máx 940 (63%)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Disponible cierres 75 cm</t>
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Remanente global al máximo</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>744</v>
+        <v>552</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Usa máx 177 (24%)</t>
+          <t>Incl. 15 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1439,14 +1449,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>★ = tienda con velocidad proyectada/ajustada</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
@@ -1530,335 +1540,335 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>SAMBIL</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="D5" s="16" t="n">
+      <c r="D5" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="16" t="n">
         <v>48</v>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="15" t="n">
         <v>42</v>
       </c>
-      <c r="G5" s="17" t="n">
+      <c r="G5" s="16" t="n">
         <v>45</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="I5" s="17" t="n">
+      <c r="I5" s="16" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="16" t="n">
+      <c r="J5" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="17" t="n">
+      <c r="K5" s="16" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>GRIETA</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="G6" s="17" t="n">
+      <c r="G6" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="I6" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="J6" s="16" t="n">
+      <c r="J6" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="17" t="n">
+      <c r="K6" s="16" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>CERRO VERDE</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="15" t="n">
         <v>29</v>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="16" t="n">
         <v>32</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="G7" s="17" t="n">
+      <c r="G7" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="I7" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="J7" s="16" t="n">
+      <c r="J7" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="K7" s="17" t="n">
+      <c r="K7" s="16" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>CHACAO</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="15" t="n">
         <v>33</v>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="16" t="n">
         <v>36</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="15" t="n">
         <v>31</v>
       </c>
-      <c r="G8" s="17" t="n">
+      <c r="G8" s="16" t="n">
         <v>35</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="15" t="n">
         <v>17</v>
       </c>
-      <c r="I8" s="17" t="n">
+      <c r="I8" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="J8" s="16" t="n">
+      <c r="J8" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="K8" s="17" t="n">
+      <c r="K8" s="16" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="18" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>GRAND PLAZ ★</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="17" t="n">
+      <c r="G9" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="16" t="n">
+      <c r="H9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="I9" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="17" t="n">
+      <c r="K9" s="16" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>LA VELA ★</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="16" t="n">
         <v>40</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="15" t="n">
         <v>34</v>
       </c>
-      <c r="G10" s="17" t="n">
+      <c r="G10" s="16" t="n">
         <v>38</v>
       </c>
-      <c r="H10" s="16" t="n">
+      <c r="H10" s="15" t="n">
         <v>19</v>
       </c>
-      <c r="I10" s="17" t="n">
+      <c r="I10" s="16" t="n">
         <v>21</v>
       </c>
-      <c r="J10" s="16" t="n">
+      <c r="J10" s="15" t="n">
         <v>5</v>
       </c>
-      <c r="K10" s="17" t="n">
+      <c r="K10" s="16" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>TOLON ★</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="16" t="n">
         <v>26</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="G11" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="I11" s="17" t="n">
+      <c r="I11" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="J11" s="16" t="n">
+      <c r="J11" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="K11" s="17" t="n">
+      <c r="K11" s="16" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>WEB ★</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="15" t="n">
         <v>12</v>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="D12" s="16" t="n">
+      <c r="D12" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="F12" s="16" t="n">
+      <c r="F12" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="H12" s="16" t="n">
+      <c r="H12" s="15" t="n">
         <v>8</v>
       </c>
-      <c r="I12" s="17" t="n">
+      <c r="I12" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="J12" s="16" t="n">
+      <c r="J12" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="17" t="n">
+      <c r="K12" s="16" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>BARQUISIMETO ★</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B13" s="15" t="n">
         <v>25</v>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="16" t="n">
         <v>27</v>
       </c>
-      <c r="D13" s="16" t="n">
+      <c r="D13" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="16" t="n">
         <v>33</v>
       </c>
-      <c r="F13" s="16" t="n">
+      <c r="F13" s="15" t="n">
         <v>28</v>
       </c>
-      <c r="G13" s="17" t="n">
+      <c r="G13" s="16" t="n">
         <v>31</v>
       </c>
-      <c r="H13" s="16" t="n">
+      <c r="H13" s="15" t="n">
         <v>16</v>
       </c>
-      <c r="I13" s="17" t="n">
+      <c r="I13" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="J13" s="16" t="n">
+      <c r="J13" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="17" t="n">
+      <c r="K13" s="16" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1900,29 +1910,29 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Totales por tienda (Mín / Máx):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="C17" s="20" t="inlineStr">
+      <c r="C17" s="19" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="D17" s="20" t="inlineStr">
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Vel. mensual proy.</t>
         </is>
@@ -2091,16 +2101,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>PLAN DE CIERRES — QX NEGRO 0580</t>
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>PLAN DE CIERRES — QX NEGRO 0580 (INVENTARIO GLOBAL)</t>
         </is>
       </c>
     </row>
@@ -2128,109 +2138,266 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="22" t="inlineStr">
-        <is>
-          <t>Longitud</t>
-        </is>
-      </c>
-      <c r="B5" s="22" t="inlineStr">
-        <is>
-          <t>Tallas</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="inlineStr">
-        <is>
-          <t>Disponible</t>
-        </is>
-      </c>
-      <c r="D5" s="22" t="inlineStr">
-        <is>
-          <t>Usa Mín</t>
-        </is>
-      </c>
-      <c r="E5" s="22" t="inlineStr">
-        <is>
-          <t>Usa Máx</t>
-        </is>
-      </c>
-      <c r="F5" s="22" t="inlineStr">
-        <is>
-          <t>Remanente Mín</t>
-        </is>
-      </c>
-      <c r="G5" s="22" t="inlineStr">
-        <is>
-          <t>Remanente Máx</t>
-        </is>
-      </c>
-      <c r="H5" s="22" t="inlineStr">
-        <is>
-          <t>% uso máx</t>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Lógica</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>75 cm adaptable a 60 cm · 1 cierre = 1 chaqueta · pool global</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>60 cm</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>XS · S · M</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>748</v>
-      </c>
-      <c r="D6" t="n">
-        <v>690</v>
-      </c>
-      <c r="E6" t="n">
-        <v>763</v>
-      </c>
-      <c r="F6" t="n">
-        <v>58</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-15</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>102%</t>
+          <t>── STOCK POR LONGITUD ──</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Longitud</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Und disponibles</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>60 cm</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>748</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Preferido XS · S · M</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>75 cm</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B9" t="n">
+        <v>744</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Preferido L · XL · adaptable a 60 cm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>TOTAL GLOBAL</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1492</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Tope producción</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>── DEMANDA POR TALLA (Mín / Máx) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Grupo</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Tallas</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Demanda Mín</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Demanda Máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>60 cm ideal</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>XS · S · M</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>690</v>
+      </c>
+      <c r="D14" t="n">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>75 cm ideal</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>L · XL</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>744</v>
-      </c>
-      <c r="D7" t="n">
+      <c r="C15" t="n">
         <v>160</v>
       </c>
-      <c r="E7" t="n">
+      <c r="D15" t="n">
         <v>177</v>
       </c>
-      <c r="F7" t="n">
-        <v>584</v>
-      </c>
-      <c r="G7" t="n">
-        <v>567</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>24%</t>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>TOTAL chaquetas</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="n">
+        <v>850</v>
+      </c>
+      <c r="D16" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>── ASIGNACIÓN AL MÁXIMO (940 und) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Und</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Cierres 60 cm usados (nativos XS/S/M)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Cierres 75 cm adaptados a 60 cm</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Cierres 75 cm usados en L/XL</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Total cierres 75 cm consumidos</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Total cierres consumidos (global)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Remanente global</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Rango producción acordado</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>850 – 940 und</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>¿Cabe en inventario global?</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SÍ</t>
         </is>
       </c>
     </row>
@@ -2245,14 +2412,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="21" t="inlineStr">
         <is>
           <t>METODOLOGÍA — PROYECCIÓN CHAQUETA LITE</t>
         </is>
@@ -2262,7 +2429,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>1. PRODUCTO DE REFERENCIA</t>
         </is>
@@ -2293,7 +2460,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>2. AJUSTE TEMPORADA ALTA</t>
         </is>
@@ -2310,7 +2477,7 @@
       <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>3. AJUSTES DE TIENDA (según indicación)</t>
         </is>
@@ -2390,7 +2557,7 @@
       <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="19" t="inlineStr">
         <is>
           <t>4. RANGO GLOBAL ACORDADO</t>
         </is>
@@ -2414,76 +2581,83 @@
       <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="inlineStr">
-        <is>
-          <t>5. INSUMO LIMITANTE — CIERRES</t>
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>5. INSUMO LIMITANTE — CIERRES (INVENTARIO GLOBAL)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Tope teórico cierres 60 cm = 921 und.</t>
+          <t xml:space="preserve">   Stock total: 748 (60 cm) + 744 (75 cm) = 1492 und.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Al máximo (940 und) se necesitan 763 cierres 60 cm.</t>
+          <t xml:space="preserve">   Los cierres 75 cm se adaptan a 60 cm → se considera pool global intercambiable.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Déficit al máximo: 15 und de cierre 60 cm (si no se compran más).</t>
+          <t xml:space="preserve">   Tope producción = 1492 und (1 cierre por chaqueta).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Al máximo (940 und) quedan 552 cierres remanentes.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>6. RANGO MÍNIMO / MÁXIMO</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Compromiso mín: 850 und.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Compromiso mín: 850 und.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Techo máx: 940 und.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="20" t="inlineStr">
+      <c r="A36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>7. DISTRIBUCIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
         </is>

</xml_diff>

<commit_message>
Subir Web a 60% Cerro Verde, Grand Plaz +20% adicional y rango 870-950 und
Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -858,7 +858,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>¿Rango 850–940 cabe en stock?</t>
+          <t>¿Rango 870–950 cabe en stock?</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>850</v>
+        <v>870</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>940</v>
+        <v>950</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -911,7 +911,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>850</v>
+        <v>870</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -941,7 +941,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>940</v>
+        <v>950</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>552</v>
+        <v>542</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1019,11 +1019,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Web proyectada (50% Cerro Verde)</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>31</v>
+        <v>37.2</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1079,11 +1079,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+40% hist.)</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>11.7</v>
+        <v>14</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1242,16 +1242,16 @@
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F5" t="n">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="G5" t="n">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6">
@@ -1269,16 +1269,16 @@
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F6" t="n">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="G6" t="n">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7">
@@ -1296,16 +1296,16 @@
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F7" t="n">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="G7" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8">
@@ -1323,16 +1323,16 @@
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F8" t="n">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="G8" t="n">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="9">
@@ -1350,16 +1350,16 @@
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F9" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G9" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10">
@@ -1369,16 +1369,16 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>850</v>
+        <v>870</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>940</v>
+        <v>950</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>690</v>
+        <v>706</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>763</v>
+        <v>770</v>
       </c>
     </row>
     <row r="12">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 940 (63%)</t>
+          <t>Usa máx 950 (64%)</t>
         </is>
       </c>
     </row>
@@ -1403,11 +1403,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>552</v>
+        <v>542</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Incl. 15 cierres 75→60 cm</t>
+          <t>Incl. 22 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
         <v>26</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" s="16" t="n">
         <v>31</v>
@@ -1604,7 +1604,7 @@
         <v>15</v>
       </c>
       <c r="I6" s="16" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J6" s="15" t="n">
         <v>3</v>
@@ -1623,7 +1623,7 @@
         <v>24</v>
       </c>
       <c r="C7" s="16" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>29</v>
@@ -1632,10 +1632,10 @@
         <v>32</v>
       </c>
       <c r="F7" s="15" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G7" s="16" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H7" s="15" t="n">
         <v>15</v>
@@ -1647,7 +1647,7 @@
         <v>4</v>
       </c>
       <c r="K7" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -1657,7 +1657,7 @@
         </is>
       </c>
       <c r="B8" s="15" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" s="16" t="n">
         <v>30</v>
@@ -1669,7 +1669,7 @@
         <v>36</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G8" s="16" t="n">
         <v>35</v>
@@ -1681,7 +1681,7 @@
         <v>19</v>
       </c>
       <c r="J8" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K8" s="16" t="n">
         <v>5</v>
@@ -1694,28 +1694,28 @@
         </is>
       </c>
       <c r="B9" s="15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="15" t="n">
         <v>6</v>
       </c>
-      <c r="E9" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="F9" s="15" t="n">
-        <v>5</v>
-      </c>
       <c r="G9" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="18" t="n">
         <v>0</v>
@@ -1743,7 +1743,7 @@
         <v>40</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G10" s="16" t="n">
         <v>38</v>
@@ -1758,7 +1758,7 @@
         <v>5</v>
       </c>
       <c r="K10" s="16" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1768,7 +1768,7 @@
         </is>
       </c>
       <c r="B11" s="15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="16" t="n">
         <v>26</v>
@@ -1783,7 +1783,7 @@
         <v>27</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H11" s="15" t="n">
         <v>15</v>
@@ -1805,34 +1805,34 @@
         </is>
       </c>
       <c r="B12" s="15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C12" s="16" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D12" s="15" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E12" s="16" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F12" s="15" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G12" s="16" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="H12" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I12" s="16" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J12" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K12" s="16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -1854,7 +1854,7 @@
         <v>33</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G13" s="16" t="n">
         <v>31</v>
@@ -1879,34 +1879,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J14" s="10" t="n">
         <v>29</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16">
@@ -1961,10 +1961,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C19" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D19" t="n">
         <v>61</v>
@@ -1977,10 +1977,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C20" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D20" t="n">
         <v>62.1</v>
@@ -1993,7 +1993,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C21" t="n">
         <v>125</v>
@@ -2009,13 +2009,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C22" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D22" t="n">
-        <v>11.7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23">
@@ -2025,10 +2025,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C23" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D23" t="n">
         <v>77.7</v>
@@ -2041,10 +2041,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C24" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -2057,13 +2057,13 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C25" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D25" t="n">
-        <v>31</v>
+        <v>37.2</v>
       </c>
     </row>
     <row r="26">
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C26" t="n">
         <v>113</v>
@@ -2260,10 +2260,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>690</v>
+        <v>706</v>
       </c>
       <c r="D14" t="n">
-        <v>763</v>
+        <v>770</v>
       </c>
     </row>
     <row r="15">
@@ -2278,10 +2278,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="D15" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16">
@@ -2292,16 +2292,16 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>850</v>
+        <v>870</v>
       </c>
       <c r="D16" t="n">
-        <v>940</v>
+        <v>950</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>── ASIGNACIÓN AL MÁXIMO (940 und) ──</t>
+          <t>── ASIGNACIÓN AL MÁXIMO (950 und) ──</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22">
@@ -2344,7 +2344,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23">
@@ -2354,7 +2354,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>192</v>
+        <v>202</v>
       </c>
     </row>
     <row r="24">
@@ -2364,7 +2364,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>940</v>
+        <v>950</v>
       </c>
     </row>
     <row r="25">
@@ -2374,7 +2374,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>552</v>
+        <v>542</v>
       </c>
     </row>
     <row r="27">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>850 – 940 und</t>
+          <t>870 – 950 und</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Web: proyectada al 50% de Cerro Verde (62 → 31 und/mes).</t>
+          <t xml:space="preserve">   • Web: proyectada al 60% de Cerro Verde (62 → 37 und/mes).</t>
         </is>
       </c>
     </row>
@@ -2528,7 +2528,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Grand Plaz: histórico × 1.4 (+40%) = 12 und/mes.</t>
+          <t xml:space="preserve">   • Grand Plaz: histórico × 1.68 (+68%) = 14 und/mes.</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2566,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mínimo: 850 und | Máximo: 940 und.</t>
+          <t xml:space="preserve">   Mínimo: 870 und | Máximo: 950 und.</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Al máximo (940 und) quedan 552 cierres remanentes.</t>
+          <t xml:space="preserve">   Al máximo (950 und) quedan 542 cierres remanentes.</t>
         </is>
       </c>
     </row>
@@ -2628,14 +2628,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Compromiso mín: 850 und.</t>
+          <t xml:space="preserve">   Compromiso mín: 870 und.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Techo máx: 940 und.</t>
+          <t xml:space="preserve">   Techo máx: 950 und.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar proyección por color (40/30/30) y compra de tela VIORI
- Nueva hoja Producción Color × Talla con Mín/Máx
- Nueva hoja Compra de Tela VIORI (mts y kg por color)
- Consumo según ficha técnica DAMA · insumos elástica/sesgo

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Producción por Talla" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Distribución por Tienda" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Cierres (Insumo)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Metodología" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Producción Color × Talla" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Compra de Tela VIORI" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Distribución por Tienda" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cierres (Insumo)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Metodología" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,6 +47,10 @@
       <i val="1"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
       <i val="1"/>
       <color rgb="00E65100"/>
     </font>
@@ -53,7 +59,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +94,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00A8C8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00424242"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B2942"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004B5320"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,28 +177,40 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -543,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -967,123 +1000,94 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
+          <t>── COLORES DE PRODUCCIÓN ──</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B40" t="n">
-        <v>8.1</v>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>und/mes</t>
+          <t>protagonista</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Vinotinto</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Web histórica</t>
-        </is>
-      </c>
-      <c r="B42" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B43" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Ver detalle</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Hoja Producción Color × Talla</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
-        </is>
-      </c>
-      <c r="B44" t="n">
-        <v>10</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B45" t="n">
-        <v>77.7</v>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Compra tela VIORI</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Hoja Compra de Tela</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Grand Plaz histórica</t>
-        </is>
-      </c>
-      <c r="B46" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>14</v>
+        <v>8.1</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1094,11 +1098,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>64.09999999999999</v>
+        <v>60.4</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1109,45 +1113,150 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>Web histórica</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Web proyectada (60% Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>37.2</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>La Vela histórica</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>10</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>Grand Plaz histórica</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>14</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
+        <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
@@ -1425,6 +1534,1032 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>CHAQUETA LITE — PRODUCCIÓN POR COLOR Y TALLA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Proporción: Negro 40% · Vinotinto 30% · Verde Militar 30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Rango global: 870 – 950 und</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Negro (40%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>84</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>101</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>111</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>96</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>105</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>53</v>
+      </c>
+      <c r="I8" s="8" t="n">
+        <v>58</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="K8" s="8" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL color</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>348</v>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="15" t="inlineStr">
+        <is>
+          <t>Vinotinto (30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="I13" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>72</v>
+      </c>
+      <c r="G14" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="I14" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="K14" s="8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL color</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>261</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Verde Militar (30%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="I19" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>63</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>69</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>76</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>83</v>
+      </c>
+      <c r="F20" s="7" t="n">
+        <v>72</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>79</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="I20" s="8" t="n">
+        <v>44</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="K20" s="8" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL color</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>261</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>870</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Resumen por color (Mín / Máx):</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>348</v>
+      </c>
+      <c r="C26" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Vinotinto</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>261</v>
+      </c>
+      <c r="C27" t="n">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>261</v>
+      </c>
+      <c r="C28" t="n">
+        <v>285</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="F6:G6"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="A11:L11"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>CHAQUETA LITE — COMPRA DE TELA VIORI POR COLOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Consumo por pieza según ficha técnica DAMA · 3 colores 40/30/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Color</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Und Mín</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Und Máx</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Metros Mín</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Metros Máx</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Kg Mín</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>Kg Máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>348</v>
+      </c>
+      <c r="D5" t="n">
+        <v>380</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>435.98</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>475.92</v>
+      </c>
+      <c r="G5" s="18" t="n">
+        <v>46.893</v>
+      </c>
+      <c r="H5" s="19" t="n">
+        <v>51.189</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Vinotinto</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>261</v>
+      </c>
+      <c r="D6" t="n">
+        <v>285</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>326.95</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>356.95</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>35.166</v>
+      </c>
+      <c r="H6" s="19" t="n">
+        <v>38.393</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>261</v>
+      </c>
+      <c r="D7" t="n">
+        <v>285</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>326.95</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>356.95</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>35.166</v>
+      </c>
+      <c r="H7" s="19" t="n">
+        <v>38.393</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL TELA VIORI</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>870</v>
+      </c>
+      <c r="D8" t="n">
+        <v>950</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>1089.88</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>1189.82</v>
+      </c>
+      <c r="G8" s="10" t="n">
+        <v>117.225</v>
+      </c>
+      <c r="H8" s="10" t="n">
+        <v>127.975</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>── DETALLE POR TALLA Y COLOR (MÁX) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Color / Talla</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Mts</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Negro</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>92</v>
+      </c>
+      <c r="C12" t="n">
+        <v>111</v>
+      </c>
+      <c r="D12" t="n">
+        <v>105</v>
+      </c>
+      <c r="E12" t="n">
+        <v>58</v>
+      </c>
+      <c r="F12" t="n">
+        <v>14</v>
+      </c>
+      <c r="G12" t="n">
+        <v>380</v>
+      </c>
+      <c r="H12" t="n">
+        <v>475.92</v>
+      </c>
+      <c r="I12" t="n">
+        <v>51.189</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Vinotinto</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>69</v>
+      </c>
+      <c r="C13" t="n">
+        <v>83</v>
+      </c>
+      <c r="D13" t="n">
+        <v>79</v>
+      </c>
+      <c r="E13" t="n">
+        <v>44</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G13" t="n">
+        <v>285</v>
+      </c>
+      <c r="H13" t="n">
+        <v>356.95</v>
+      </c>
+      <c r="I13" t="n">
+        <v>38.393</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Verde Militar</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>69</v>
+      </c>
+      <c r="C14" t="n">
+        <v>83</v>
+      </c>
+      <c r="D14" t="n">
+        <v>79</v>
+      </c>
+      <c r="E14" t="n">
+        <v>44</v>
+      </c>
+      <c r="F14" t="n">
+        <v>10</v>
+      </c>
+      <c r="G14" t="n">
+        <v>285</v>
+      </c>
+      <c r="H14" t="n">
+        <v>356.95</v>
+      </c>
+      <c r="I14" t="n">
+        <v>38.393</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>── CONSUMO UNITARIO VIORI (referencia ficha) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Talla</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Metros/pieza</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1.22</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Kg/pieza</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.138</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.144</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.145</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>── OTROS INSUMOS (total producción Mín / Máx) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Elástica 4.5 cm (metros)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>430.19</v>
+      </c>
+      <c r="C22" t="n">
+        <v>469.78</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sesgo cintura 2 cm (metros)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>464.99</v>
+      </c>
+      <c r="C23" t="n">
+        <v>507.78</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sesgo manga 2 cm (metros)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>169.19</v>
+      </c>
+      <c r="C24" t="n">
+        <v>184.78</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1449,7 +2584,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>★ = tienda con velocidad proyectada/ajustada</t>
         </is>
@@ -1540,335 +2675,335 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>SAMBIL</t>
         </is>
       </c>
-      <c r="B5" s="15" t="n">
+      <c r="B5" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="18" t="n">
         <v>44</v>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="19" t="n">
         <v>48</v>
       </c>
-      <c r="F5" s="15" t="n">
+      <c r="F5" s="18" t="n">
         <v>42</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="G5" s="19" t="n">
         <v>45</v>
       </c>
-      <c r="H5" s="15" t="n">
+      <c r="H5" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="I5" s="16" t="n">
+      <c r="I5" s="19" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="J5" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="16" t="n">
+      <c r="K5" s="19" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>GRIETA</t>
         </is>
       </c>
-      <c r="B6" s="15" t="n">
+      <c r="B6" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="F6" s="15" t="n">
+      <c r="F6" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="H6" s="15" t="n">
+      <c r="H6" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="J6" s="15" t="n">
+      <c r="J6" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K6" s="16" t="n">
+      <c r="K6" s="19" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>CERRO VERDE</t>
         </is>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="19" t="n">
         <v>32</v>
       </c>
-      <c r="F7" s="15" t="n">
+      <c r="F7" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="H7" s="15" t="n">
+      <c r="H7" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="I7" s="16" t="n">
+      <c r="I7" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J7" s="15" t="n">
+      <c r="J7" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="K7" s="16" t="n">
+      <c r="K7" s="19" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>CHACAO</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="19" t="n">
         <v>30</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="18" t="n">
         <v>33</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="19" t="n">
         <v>36</v>
       </c>
-      <c r="F8" s="15" t="n">
+      <c r="F8" s="18" t="n">
         <v>32</v>
       </c>
-      <c r="G8" s="16" t="n">
+      <c r="G8" s="19" t="n">
         <v>35</v>
       </c>
-      <c r="H8" s="15" t="n">
+      <c r="H8" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="I8" s="16" t="n">
+      <c r="I8" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="J8" s="15" t="n">
+      <c r="J8" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="K8" s="16" t="n">
+      <c r="K8" s="19" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>GRAND PLAZ ★</t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="19" t="n">
         <v>6</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="G9" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="16" t="n">
+      <c r="I9" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="J9" s="18" t="n">
+      <c r="J9" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="K9" s="16" t="n">
+      <c r="K9" s="19" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>LA VELA ★</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="19" t="n">
         <v>33</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="19" t="n">
         <v>40</v>
       </c>
-      <c r="F10" s="15" t="n">
+      <c r="F10" s="18" t="n">
         <v>35</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="19" t="n">
         <v>38</v>
       </c>
-      <c r="H10" s="15" t="n">
+      <c r="H10" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="I10" s="16" t="n">
+      <c r="I10" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="J10" s="15" t="n">
+      <c r="J10" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="K10" s="16" t="n">
+      <c r="K10" s="19" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>TOLON ★</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="18" t="n">
         <v>24</v>
       </c>
-      <c r="C11" s="16" t="n">
+      <c r="C11" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="F11" s="15" t="n">
+      <c r="F11" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="19" t="n">
         <v>29</v>
       </c>
-      <c r="H11" s="15" t="n">
+      <c r="H11" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="I11" s="16" t="n">
+      <c r="I11" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="J11" s="15" t="n">
+      <c r="J11" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K11" s="16" t="n">
+      <c r="K11" s="19" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>WEB ★</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="18" t="n">
         <v>15</v>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="E12" s="16" t="n">
+      <c r="E12" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="F12" s="15" t="n">
+      <c r="F12" s="18" t="n">
         <v>17</v>
       </c>
-      <c r="G12" s="16" t="n">
+      <c r="G12" s="19" t="n">
         <v>18</v>
       </c>
-      <c r="H12" s="15" t="n">
+      <c r="H12" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I12" s="16" t="n">
+      <c r="I12" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="J12" s="15" t="n">
+      <c r="J12" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="K12" s="16" t="n">
+      <c r="K12" s="19" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>BARQUISIMETO ★</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="18" t="n">
         <v>25</v>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="19" t="n">
         <v>27</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="18" t="n">
         <v>30</v>
       </c>
-      <c r="E13" s="16" t="n">
+      <c r="E13" s="19" t="n">
         <v>33</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="F13" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="G13" s="16" t="n">
+      <c r="G13" s="19" t="n">
         <v>31</v>
       </c>
-      <c r="H13" s="15" t="n">
+      <c r="H13" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="I13" s="16" t="n">
+      <c r="I13" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="J13" s="15" t="n">
+      <c r="J13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="K13" s="16" t="n">
+      <c r="K13" s="19" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1910,29 +3045,29 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Totales por tienda (Mín / Máx):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="C17" s="19" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Vel. mensual proy.</t>
         </is>
@@ -2095,7 +3230,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2108,7 +3243,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="20" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>PLAN DE CIERRES — QX NEGRO 0580 (INVENTARIO GLOBAL)</t>
         </is>
@@ -2406,20 +3541,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t>METODOLOGÍA — PROYECCIÓN CHAQUETA LITE</t>
         </is>
@@ -2429,7 +3564,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>1. PRODUCTO DE REFERENCIA</t>
         </is>
@@ -2460,7 +3595,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>2. AJUSTE TEMPORADA ALTA</t>
         </is>
@@ -2477,7 +3612,7 @@
       <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>3. AJUSTES DE TIENDA (según indicación)</t>
         </is>
@@ -2557,7 +3692,7 @@
       <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="19" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>4. RANGO GLOBAL ACORDADO</t>
         </is>
@@ -2581,7 +3716,7 @@
       <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>5. INSUMO LIMITANTE — CIERRES (INVENTARIO GLOBAL)</t>
         </is>
@@ -2619,7 +3754,7 @@
       <c r="A32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="19" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>6. RANGO MÍNIMO / MÁXIMO</t>
         </is>
@@ -2643,7 +3778,7 @@
       <c r="A36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="19" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>7. DISTRIBUCIÓN</t>
         </is>
@@ -2660,6 +3795,44 @@
       <c r="A39" t="inlineStr">
         <is>
           <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>8. COLORES Y COMPRA DE TELA</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregar hoja Cantidades por Colores (curva SPOTS) y rango 890-970
- Pestaña con curva completa color×talla Mín/Máx estilo SPOTS
- Insumos integrados: tela VIORI, elástica, sesgos, cierres
- Rango global actualizado a 890–970 und

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet name="Resumen" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Producción por Talla" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Producción Color × Talla" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Compra de Tela VIORI" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Distribución por Tienda" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Cierres (Insumo)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Metodología" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cantidades por Colores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Producción Color × Talla" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Compra de Tela VIORI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Distribución por Tienda" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Cierres (Insumo)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Metodología" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,6 +49,34 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
     <font>
@@ -59,7 +88,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -98,6 +127,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4BC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00A9D08E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00424242"/>
       </patternFill>
     </fill>
@@ -109,11 +158,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="004B5320"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -148,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,40 +221,65 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -576,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -891,7 +960,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>¿Rango 870–950 cabe en stock?</t>
+          <t>¿Rango 890–970 cabe en stock?</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -914,7 +983,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>870</v>
+        <v>890</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -929,7 +998,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>950</v>
+        <v>970</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -959,7 +1028,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>870</v>
+        <v>890</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -974,7 +1043,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>950</v>
+        <v>970</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -989,7 +1058,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>542</v>
+        <v>522</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1050,12 +1119,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Ver detalle</t>
+          <t>Curva completa color × talla</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Hoja Producción Color × Talla</t>
+          <t>Hoja Cantidades por Colores</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1063,46 +1132,44 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>Detalle color/talla Mín-Máx</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Hoja Producción Color × Talla</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>Compra tela VIORI</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>Hoja Compra de Tela</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B47" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>60.4</v>
+        <v>8.1</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1113,11 +1180,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Web histórica</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>7.8</v>
+        <v>60.4</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1128,11 +1195,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>37.2</v>
+        <v>7.8</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1143,11 +1210,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>10</v>
+        <v>37.2</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1158,11 +1225,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>77.7</v>
+        <v>10</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1173,11 +1240,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>8.300000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1188,11 +1255,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>Grand Plaz histórica</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>14</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1203,11 +1270,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>64.09999999999999</v>
+        <v>14</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1218,45 +1285,60 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>Corporativo</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>EXCLUIDO</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
@@ -1351,16 +1433,16 @@
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="F5" t="n">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="G5" t="n">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6">
@@ -1378,16 +1460,16 @@
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="F6" t="n">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="G6" t="n">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="7">
@@ -1405,16 +1487,16 @@
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F7" t="n">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="G7" t="n">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8">
@@ -1432,16 +1514,16 @@
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F8" t="n">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G8" t="n">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9">
@@ -1459,13 +1541,13 @@
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E9" s="8" t="n">
         <v>35</v>
       </c>
       <c r="F9" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G9" t="n">
         <v>35</v>
@@ -1478,16 +1560,16 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>870</v>
+        <v>890</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>950</v>
+        <v>970</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>706</v>
+        <v>722</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>770</v>
+        <v>787</v>
       </c>
     </row>
     <row r="12">
@@ -1501,7 +1583,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 950 (64%)</t>
+          <t>Usa máx 970 (65%)</t>
         </is>
       </c>
     </row>
@@ -1512,11 +1594,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>542</v>
+        <v>522</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Incl. 22 cierres 75→60 cm</t>
+          <t>Incl. 39 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1529,6 +1611,607 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>CANTIDADES POR COLORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>CHAQUETA LITE · Proporción Negro 40% · Vinotinto 30% · Verde Militar 30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Rango producción: 890 – 970 und</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>MÍNIMO — 890 und (compromiso)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>CHAQUETA LITE DAMA</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E6" s="16" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G6" s="16" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Negro · 40%</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="n">
+        <v>86</v>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>104</v>
+      </c>
+      <c r="D7" s="18" t="n">
+        <v>99</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>Vinotinto · 30%</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="n">
+        <v>65</v>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>78</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>74</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>41</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>Verde Militar · 30%</t>
+        </is>
+      </c>
+      <c r="B9" s="18" t="n">
+        <v>65</v>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>78</v>
+      </c>
+      <c r="D9" s="18" t="n">
+        <v>74</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>41</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B10" s="20" t="n">
+        <v>216</v>
+      </c>
+      <c r="C10" s="20" t="n">
+        <v>260</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>247</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>136</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>31</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>MÁXIMO — 970 und (techo)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>CHAQUETA LITE DAMA</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G13" s="16" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>Negro · 40%</t>
+        </is>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>94</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>113</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>108</v>
+      </c>
+      <c r="E14" s="18" t="n">
+        <v>59</v>
+      </c>
+      <c r="F14" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="G14" s="18" t="n">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Vinotinto · 30%</t>
+        </is>
+      </c>
+      <c r="B15" s="18" t="n">
+        <v>71</v>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>81</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Verde Militar · 30%</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>71</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>85</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>81</v>
+      </c>
+      <c r="E16" s="18" t="n">
+        <v>44</v>
+      </c>
+      <c r="F16" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" s="18" t="n">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="n">
+        <v>236</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>283</v>
+      </c>
+      <c r="D17" s="20" t="n">
+        <v>270</v>
+      </c>
+      <c r="E17" s="20" t="n">
+        <v>147</v>
+      </c>
+      <c r="F17" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="G17" s="20" t="n">
+        <v>970</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>── INSUMOS PARA COMPRA (Mín / Máx) ──</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Insumo</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>Tela VIORI — Negro</t>
+        </is>
+      </c>
+      <c r="B21" s="23" t="n">
+        <v>445.85</v>
+      </c>
+      <c r="C21" s="24" t="n">
+        <v>485.92</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>52.265 kg al máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="inlineStr">
+        <is>
+          <t>Tela VIORI — Vinotinto</t>
+        </is>
+      </c>
+      <c r="B22" s="23" t="n">
+        <v>334.32</v>
+      </c>
+      <c r="C22" s="24" t="n">
+        <v>364.33</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>39.187 kg al máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>Tela VIORI — Verde Militar</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="n">
+        <v>334.32</v>
+      </c>
+      <c r="C23" s="24" t="n">
+        <v>364.33</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>39.187 kg al máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="inlineStr">
+        <is>
+          <t>TOTAL tela VIORI</t>
+        </is>
+      </c>
+      <c r="B24" s="23" t="n">
+        <v>1114.49</v>
+      </c>
+      <c r="C24" s="24" t="n">
+        <v>1214.58</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>130.639 kg al máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="inlineStr">
+        <is>
+          <t>Elástica 4.5 cm</t>
+        </is>
+      </c>
+      <c r="B25" s="23" t="n">
+        <v>440.09</v>
+      </c>
+      <c r="C25" s="24" t="n">
+        <v>479.65</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Ficha técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="inlineStr">
+        <is>
+          <t>Sesgo cintura 2 cm</t>
+        </is>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>475.69</v>
+      </c>
+      <c r="C26" s="24" t="n">
+        <v>518.45</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Ficha técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="inlineStr">
+        <is>
+          <t>Sesgo manga 2 cm</t>
+        </is>
+      </c>
+      <c r="B27" s="23" t="n">
+        <v>173.09</v>
+      </c>
+      <c r="C27" s="24" t="n">
+        <v>188.65</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Ficha técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>Cierres QX Negro 0580</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="n">
+        <v>890</v>
+      </c>
+      <c r="C28" s="24" t="n">
+        <v>970</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Pool global 1492 und · rem. 522 al máx</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · Preferencia 60 cm (XS/S/M)</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="n">
+        <v>722</v>
+      </c>
+      <c r="C29" s="26" t="n">
+        <v>787</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Stock 748 und</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · Preferencia 75 cm (L/XL)</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="n">
+        <v>168</v>
+      </c>
+      <c r="C30" s="26" t="n">
+        <v>183</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Stock 744 und · adaptable</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A6"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A12:G12"/>
+    <mergeCell ref="A13"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1567,19 +2250,19 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Rango global: 870 – 950 und</t>
+          <t>Rango global: 890 – 970 und</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Negro (40%)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
@@ -1663,37 +2346,37 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K8" s="8" t="n">
         <v>14</v>
@@ -1706,21 +2389,21 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Vinotinto (30%)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
@@ -1804,37 +2487,37 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I14" s="8" t="n">
         <v>44</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K14" s="8" t="n">
         <v>10</v>
@@ -1847,21 +2530,21 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>Verde Militar (30%)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="28" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
@@ -1945,37 +2628,37 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>Cantidad</t>
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I20" s="8" t="n">
         <v>44</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K20" s="8" t="n">
         <v>10</v>
@@ -1988,10 +2671,10 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="23">
@@ -2001,14 +2684,14 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>870</v>
+        <v>890</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>950</v>
+        <v>970</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Resumen por color (Mín / Máx):</t>
         </is>
@@ -2021,10 +2704,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="C26" t="n">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="27">
@@ -2034,10 +2717,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="C27" t="n">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="28">
@@ -2047,10 +2730,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="C28" t="n">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -2079,7 +2762,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2156,7 +2839,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Negro</t>
         </is>
@@ -2167,26 +2850,26 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="D5" t="n">
-        <v>380</v>
-      </c>
-      <c r="E5" s="18" t="n">
-        <v>435.98</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>475.92</v>
-      </c>
-      <c r="G5" s="18" t="n">
-        <v>46.893</v>
-      </c>
-      <c r="H5" s="19" t="n">
-        <v>51.189</v>
+        <v>388</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>445.85</v>
+      </c>
+      <c r="F5" s="24" t="n">
+        <v>485.92</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>47.955</v>
+      </c>
+      <c r="H5" s="24" t="n">
+        <v>52.265</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Vinotinto</t>
         </is>
@@ -2197,26 +2880,26 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="D6" t="n">
-        <v>285</v>
-      </c>
-      <c r="E6" s="18" t="n">
-        <v>326.95</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>356.95</v>
-      </c>
-      <c r="G6" s="18" t="n">
-        <v>35.166</v>
-      </c>
-      <c r="H6" s="19" t="n">
-        <v>38.393</v>
+        <v>291</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>334.32</v>
+      </c>
+      <c r="F6" s="24" t="n">
+        <v>364.33</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>35.959</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <v>39.187</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>Verde Militar</t>
         </is>
@@ -2227,22 +2910,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="D7" t="n">
-        <v>285</v>
-      </c>
-      <c r="E7" s="18" t="n">
-        <v>326.95</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>356.95</v>
-      </c>
-      <c r="G7" s="18" t="n">
-        <v>35.166</v>
-      </c>
-      <c r="H7" s="19" t="n">
-        <v>38.393</v>
+        <v>291</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <v>334.32</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>364.33</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>35.959</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <v>39.187</v>
       </c>
     </row>
     <row r="8">
@@ -2252,26 +2935,26 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>870</v>
+        <v>890</v>
       </c>
       <c r="D8" t="n">
-        <v>950</v>
+        <v>970</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>1089.88</v>
+        <v>1114.49</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>1189.82</v>
+        <v>1214.58</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>117.225</v>
+        <v>119.873</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>127.975</v>
+        <v>130.639</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>── DETALLE POR TALLA Y COLOR (MÁX) ──</t>
         </is>
@@ -2325,50 +3008,50 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="27" t="inlineStr">
         <is>
           <t>Negro</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C12" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D12" t="n">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="E12" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F12" t="n">
         <v>14</v>
       </c>
       <c r="G12" t="n">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="H12" t="n">
-        <v>475.92</v>
+        <v>485.92</v>
       </c>
       <c r="I12" t="n">
-        <v>51.189</v>
+        <v>52.265</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>Vinotinto</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C13" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D13" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E13" t="n">
         <v>44</v>
@@ -2377,29 +3060,29 @@
         <v>10</v>
       </c>
       <c r="G13" t="n">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="H13" t="n">
-        <v>356.95</v>
+        <v>364.33</v>
       </c>
       <c r="I13" t="n">
-        <v>38.393</v>
+        <v>39.187</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>Verde Militar</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C14" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D14" t="n">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E14" t="n">
         <v>44</v>
@@ -2408,24 +3091,24 @@
         <v>10</v>
       </c>
       <c r="G14" t="n">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="H14" t="n">
-        <v>356.95</v>
+        <v>364.33</v>
       </c>
       <c r="I14" t="n">
-        <v>38.393</v>
+        <v>39.187</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>── CONSUMO UNITARIO VIORI (referencia ficha) ──</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>Talla</t>
         </is>
@@ -2501,7 +3184,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>── OTROS INSUMOS (total producción Mín / Máx) ──</t>
         </is>
@@ -2514,10 +3197,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>430.19</v>
+        <v>440.09</v>
       </c>
       <c r="C22" t="n">
-        <v>469.78</v>
+        <v>479.65</v>
       </c>
     </row>
     <row r="23">
@@ -2527,10 +3210,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>464.99</v>
+        <v>475.69</v>
       </c>
       <c r="C23" t="n">
-        <v>507.78</v>
+        <v>518.45</v>
       </c>
     </row>
     <row r="24">
@@ -2540,10 +3223,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>169.19</v>
+        <v>173.09</v>
       </c>
       <c r="C24" t="n">
-        <v>184.78</v>
+        <v>188.65</v>
       </c>
     </row>
   </sheetData>
@@ -2554,7 +3237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2584,14 +3267,14 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>★ = tienda con velocidad proyectada/ajustada</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
@@ -2675,336 +3358,336 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>SAMBIL</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
-        <v>36</v>
-      </c>
-      <c r="C5" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="D5" s="18" t="n">
-        <v>44</v>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>48</v>
-      </c>
-      <c r="F5" s="18" t="n">
-        <v>42</v>
-      </c>
-      <c r="G5" s="19" t="n">
+      <c r="B5" s="23" t="n">
+        <v>37</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>41</v>
+      </c>
+      <c r="D5" s="23" t="n">
         <v>45</v>
       </c>
-      <c r="H5" s="18" t="n">
-        <v>23</v>
-      </c>
-      <c r="I5" s="19" t="n">
+      <c r="E5" s="24" t="n">
+        <v>49</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>43</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>47</v>
+      </c>
+      <c r="H5" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="I5" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="J5" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" s="24" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="inlineStr">
+        <is>
+          <t>GRIETA</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>29</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>32</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="I6" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="J6" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K6" s="24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>CERRO VERDE</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
         <v>25</v>
       </c>
-      <c r="J5" s="18" t="n">
+      <c r="C7" s="24" t="n">
+        <v>27</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>32</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>31</v>
+      </c>
+      <c r="H7" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="I7" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="J7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>CHACAO</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>31</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>34</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>37</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>35</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="I8" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="J8" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="K5" s="19" t="n">
+      <c r="K8" s="24" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="32" t="inlineStr">
+        <is>
+          <t>GRAND PLAZ ★</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>GRIETA</t>
-        </is>
-      </c>
-      <c r="B6" s="18" t="n">
+      <c r="C9" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>7</v>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>LA VELA ★</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n">
+        <v>31</v>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>34</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>37</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>41</v>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>39</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" s="24" t="n">
+        <v>21</v>
+      </c>
+      <c r="J10" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" s="24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>TOLON ★</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n">
         <v>24</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C11" s="24" t="n">
         <v>26</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D11" s="23" t="n">
         <v>29</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E11" s="24" t="n">
         <v>31</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F11" s="23" t="n">
         <v>27</v>
       </c>
-      <c r="G6" s="19" t="n">
+      <c r="G11" s="24" t="n">
         <v>30</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H11" s="23" t="n">
         <v>15</v>
       </c>
-      <c r="I6" s="19" t="n">
+      <c r="I11" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="J11" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="24" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>WEB ★</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="C12" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="J6" s="18" t="n">
+      <c r="D12" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="F12" s="23" t="n">
+        <v>17</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>19</v>
+      </c>
+      <c r="H12" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="I12" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="J12" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" s="24" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>BARQUISIMETO ★</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="C13" s="24" t="n">
+        <v>28</v>
+      </c>
+      <c r="D13" s="23" t="n">
+        <v>31</v>
+      </c>
+      <c r="E13" s="24" t="n">
+        <v>34</v>
+      </c>
+      <c r="F13" s="23" t="n">
+        <v>29</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>32</v>
+      </c>
+      <c r="H13" s="23" t="n">
+        <v>16</v>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>18</v>
+      </c>
+      <c r="J13" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" s="24" t="n">
         <v>3</v>
-      </c>
-      <c r="K6" s="19" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>CERRO VERDE</t>
-        </is>
-      </c>
-      <c r="B7" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="C7" s="19" t="n">
-        <v>26</v>
-      </c>
-      <c r="D7" s="18" t="n">
-        <v>29</v>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>32</v>
-      </c>
-      <c r="F7" s="18" t="n">
-        <v>28</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>30</v>
-      </c>
-      <c r="H7" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="I7" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="J7" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="19" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="21" t="inlineStr">
-        <is>
-          <t>CHACAO</t>
-        </is>
-      </c>
-      <c r="B8" s="18" t="n">
-        <v>28</v>
-      </c>
-      <c r="C8" s="19" t="n">
-        <v>30</v>
-      </c>
-      <c r="D8" s="18" t="n">
-        <v>33</v>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>36</v>
-      </c>
-      <c r="F8" s="18" t="n">
-        <v>32</v>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>35</v>
-      </c>
-      <c r="H8" s="18" t="n">
-        <v>17</v>
-      </c>
-      <c r="I8" s="19" t="n">
-        <v>19</v>
-      </c>
-      <c r="J8" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="19" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="22" t="inlineStr">
-        <is>
-          <t>GRAND PLAZ ★</t>
-        </is>
-      </c>
-      <c r="B9" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="C9" s="19" t="n">
-        <v>6</v>
-      </c>
-      <c r="D9" s="18" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="H9" s="18" t="n">
-        <v>4</v>
-      </c>
-      <c r="I9" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="J9" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="19" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>LA VELA ★</t>
-        </is>
-      </c>
-      <c r="B10" s="18" t="n">
-        <v>30</v>
-      </c>
-      <c r="C10" s="19" t="n">
-        <v>33</v>
-      </c>
-      <c r="D10" s="18" t="n">
-        <v>36</v>
-      </c>
-      <c r="E10" s="19" t="n">
-        <v>40</v>
-      </c>
-      <c r="F10" s="18" t="n">
-        <v>35</v>
-      </c>
-      <c r="G10" s="19" t="n">
-        <v>38</v>
-      </c>
-      <c r="H10" s="18" t="n">
-        <v>19</v>
-      </c>
-      <c r="I10" s="19" t="n">
-        <v>21</v>
-      </c>
-      <c r="J10" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="K10" s="19" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t>TOLON ★</t>
-        </is>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>24</v>
-      </c>
-      <c r="C11" s="19" t="n">
-        <v>26</v>
-      </c>
-      <c r="D11" s="18" t="n">
-        <v>28</v>
-      </c>
-      <c r="E11" s="19" t="n">
-        <v>31</v>
-      </c>
-      <c r="F11" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="G11" s="19" t="n">
-        <v>29</v>
-      </c>
-      <c r="H11" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="I11" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="J11" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="K11" s="19" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t>WEB ★</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="C12" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="D12" s="18" t="n">
-        <v>17</v>
-      </c>
-      <c r="E12" s="19" t="n">
-        <v>19</v>
-      </c>
-      <c r="F12" s="18" t="n">
-        <v>17</v>
-      </c>
-      <c r="G12" s="19" t="n">
-        <v>18</v>
-      </c>
-      <c r="H12" s="18" t="n">
-        <v>9</v>
-      </c>
-      <c r="I12" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="J12" s="18" t="n">
-        <v>2</v>
-      </c>
-      <c r="K12" s="19" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr">
-        <is>
-          <t>BARQUISIMETO ★</t>
-        </is>
-      </c>
-      <c r="B13" s="18" t="n">
-        <v>25</v>
-      </c>
-      <c r="C13" s="19" t="n">
-        <v>27</v>
-      </c>
-      <c r="D13" s="18" t="n">
-        <v>30</v>
-      </c>
-      <c r="E13" s="19" t="n">
-        <v>33</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>29</v>
-      </c>
-      <c r="G13" s="19" t="n">
-        <v>31</v>
-      </c>
-      <c r="H13" s="18" t="n">
-        <v>16</v>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>17</v>
-      </c>
-      <c r="J13" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="19" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="14">
@@ -3014,60 +3697,60 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="17" t="inlineStr">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>Totales por tienda (Mín / Máx):</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Tienda</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="D17" s="17" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Vel. mensual proy.</t>
         </is>
@@ -3080,10 +3763,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C18" t="n">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D18" t="n">
         <v>93.3</v>
@@ -3096,10 +3779,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C19" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D19" t="n">
         <v>61</v>
@@ -3112,10 +3795,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C20" t="n">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D20" t="n">
         <v>62.1</v>
@@ -3128,10 +3811,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C21" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D21" t="n">
         <v>71</v>
@@ -3160,10 +3843,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C23" t="n">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D23" t="n">
         <v>77.7</v>
@@ -3176,10 +3859,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C24" t="n">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -3192,10 +3875,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C25" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D25" t="n">
         <v>37.2</v>
@@ -3208,10 +3891,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C26" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D26" t="n">
         <v>64.09999999999999</v>
@@ -3230,7 +3913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3243,7 +3926,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="24" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>PLAN DE CIERRES — QX NEGRO 0580 (INVENTARIO GLOBAL)</t>
         </is>
@@ -3395,10 +4078,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>706</v>
+        <v>722</v>
       </c>
       <c r="D14" t="n">
-        <v>770</v>
+        <v>787</v>
       </c>
     </row>
     <row r="15">
@@ -3413,10 +4096,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D15" t="n">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16">
@@ -3427,16 +4110,16 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>870</v>
+        <v>890</v>
       </c>
       <c r="D16" t="n">
-        <v>950</v>
+        <v>970</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>── ASIGNACIÓN AL MÁXIMO (950 und) ──</t>
+          <t>── ASIGNACIÓN AL MÁXIMO (970 und) ──</t>
         </is>
       </c>
     </row>
@@ -3469,7 +4152,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22">
@@ -3479,7 +4162,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23">
@@ -3489,7 +4172,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>202</v>
+        <v>222</v>
       </c>
     </row>
     <row r="24">
@@ -3499,7 +4182,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>950</v>
+        <v>970</v>
       </c>
     </row>
     <row r="25">
@@ -3509,7 +4192,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>542</v>
+        <v>522</v>
       </c>
     </row>
     <row r="27">
@@ -3520,7 +4203,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>870 – 950 und</t>
+          <t>890 – 970 und</t>
         </is>
       </c>
     </row>
@@ -3541,7 +4224,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3554,7 +4237,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="34" t="inlineStr">
         <is>
           <t>METODOLOGÍA — PROYECCIÓN CHAQUETA LITE</t>
         </is>
@@ -3564,7 +4247,7 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="17" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>1. PRODUCTO DE REFERENCIA</t>
         </is>
@@ -3595,7 +4278,7 @@
       <c r="A7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>2. AJUSTE TEMPORADA ALTA</t>
         </is>
@@ -3612,7 +4295,7 @@
       <c r="A10" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>3. AJUSTES DE TIENDA (según indicación)</t>
         </is>
@@ -3692,7 +4375,7 @@
       <c r="A22" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>4. RANGO GLOBAL ACORDADO</t>
         </is>
@@ -3701,7 +4384,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mínimo: 870 und | Máximo: 950 und.</t>
+          <t xml:space="preserve">   Mínimo: 890 und | Máximo: 970 und.</t>
         </is>
       </c>
     </row>
@@ -3716,7 +4399,7 @@
       <c r="A26" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>5. INSUMO LIMITANTE — CIERRES (INVENTARIO GLOBAL)</t>
         </is>
@@ -3746,7 +4429,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Al máximo (950 und) quedan 542 cierres remanentes.</t>
+          <t xml:space="preserve">   Al máximo (970 und) quedan 522 cierres remanentes.</t>
         </is>
       </c>
     </row>
@@ -3754,7 +4437,7 @@
       <c r="A32" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>6. RANGO MÍNIMO / MÁXIMO</t>
         </is>
@@ -3763,14 +4446,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Compromiso mín: 870 und.</t>
+          <t xml:space="preserve">   Compromiso mín: 890 und.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Techo máx: 950 und.</t>
+          <t xml:space="preserve">   Techo máx: 970 und.</t>
         </is>
       </c>
     </row>
@@ -3778,7 +4461,7 @@
       <c r="A36" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="17" t="inlineStr">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>7. DISTRIBUCIÓN</t>
         </is>
@@ -3802,7 +4485,7 @@
       <c r="A40" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="17" t="inlineStr">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>8. COLORES Y COMPRA DE TELA</t>
         </is>

</xml_diff>

<commit_message>
Agregar stock de seguridad +20% en compra de tela VIORI
- TELA_SS_PCT = 0.20 aplicado sobre consumo por color
- Hojas Compra de Tela y Cantidades por Colores muestran consumo vs compra
- Metodología y salida del script documentan totales con SS

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Hoja Compra de Tela</t>
+          <t>Hoja Compra de Tela (+20% SS)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr"/>
@@ -1616,7 +1616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1972,7 +1972,7 @@
     <row r="21">
       <c r="A21" s="22" t="inlineStr">
         <is>
-          <t>Tela VIORI — Negro</t>
+          <t>Tela VIORI — Negro (consumo)</t>
         </is>
       </c>
       <c r="B21" s="23" t="n">
@@ -1988,21 +1988,21 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>52.265 kg al máx</t>
+          <t>Sin SS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="22" t="inlineStr">
         <is>
-          <t>Tela VIORI — Vinotinto</t>
+          <t>Tela VIORI — Negro (compra +SS)</t>
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>334.32</v>
+        <v>535.02</v>
       </c>
       <c r="C22" s="24" t="n">
-        <v>364.33</v>
+        <v>583.1</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2011,21 +2011,21 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>39.187 kg al máx</t>
+          <t>62.718 kg al máx</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="22" t="inlineStr">
         <is>
-          <t>Tela VIORI — Verde Militar</t>
+          <t>Tela VIORI — Vinotinto (compra +SS)</t>
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>334.32</v>
+        <v>401.18</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>364.33</v>
+        <v>437.2</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2034,21 +2034,21 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>39.187 kg al máx</t>
+          <t>47.024 kg al máx</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>TOTAL tela VIORI</t>
+          <t>Tela VIORI — Verde Militar (compra +SS)</t>
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>1114.49</v>
+        <v>401.18</v>
       </c>
       <c r="C24" s="24" t="n">
-        <v>1214.58</v>
+        <v>437.2</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2057,21 +2057,21 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>130.639 kg al máx</t>
+          <t>47.024 kg al máx</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="22" t="inlineStr">
         <is>
-          <t>Elástica 4.5 cm</t>
+          <t>TOTAL tela VIORI (compra +SS)</t>
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>440.09</v>
+        <v>1337.39</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>479.65</v>
+        <v>1457.5</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2080,21 +2080,21 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ficha técnica</t>
+          <t>156.767 kg al máx · SS 20%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>Sesgo cintura 2 cm</t>
+          <t>Elástica 4.5 cm</t>
         </is>
       </c>
       <c r="B26" s="23" t="n">
-        <v>475.69</v>
+        <v>440.09</v>
       </c>
       <c r="C26" s="24" t="n">
-        <v>518.45</v>
+        <v>479.65</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2110,14 +2110,14 @@
     <row r="27">
       <c r="A27" s="22" t="inlineStr">
         <is>
-          <t>Sesgo manga 2 cm</t>
+          <t>Sesgo cintura 2 cm</t>
         </is>
       </c>
       <c r="B27" s="23" t="n">
-        <v>173.09</v>
+        <v>475.69</v>
       </c>
       <c r="C27" s="24" t="n">
-        <v>188.65</v>
+        <v>518.45</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2133,67 +2133,90 @@
     <row r="28">
       <c r="A28" s="22" t="inlineStr">
         <is>
+          <t>Sesgo manga 2 cm</t>
+        </is>
+      </c>
+      <c r="B28" s="23" t="n">
+        <v>173.09</v>
+      </c>
+      <c r="C28" s="24" t="n">
+        <v>188.65</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>metros</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Ficha técnica</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
           <t>Cierres QX Negro 0580</t>
         </is>
       </c>
-      <c r="B28" s="23" t="n">
+      <c r="B29" s="23" t="n">
         <v>890</v>
       </c>
-      <c r="C28" s="24" t="n">
+      <c r="C29" s="24" t="n">
         <v>970</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Pool global 1492 und · rem. 522 al máx</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · Preferencia 60 cm (XS/S/M)</t>
-        </is>
-      </c>
-      <c r="B29" s="26" t="n">
-        <v>722</v>
-      </c>
-      <c r="C29" s="26" t="n">
-        <v>787</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>Stock 748 und</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="25" t="inlineStr">
         <is>
+          <t xml:space="preserve">  · Preferencia 60 cm (XS/S/M)</t>
+        </is>
+      </c>
+      <c r="B30" s="26" t="n">
+        <v>722</v>
+      </c>
+      <c r="C30" s="26" t="n">
+        <v>787</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Stock 748 und</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  · Preferencia 75 cm (L/XL)</t>
         </is>
       </c>
-      <c r="B30" s="26" t="n">
+      <c r="B31" s="26" t="n">
         <v>168</v>
       </c>
-      <c r="C30" s="26" t="n">
+      <c r="C31" s="26" t="n">
         <v>183</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Stock 744 und · adaptable</t>
         </is>
@@ -2768,7 +2791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2792,7 +2815,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Consumo por pieza según ficha técnica DAMA · 3 colores 40/30/30</t>
+          <t>Consumo ficha técnica DAMA · 3 colores 40/30/30 · SS tela +20%</t>
         </is>
       </c>
     </row>
@@ -2819,22 +2842,32 @@
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Metros Mín</t>
+          <t>Mts consumo Mín</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Metros Máx</t>
+          <t>Mts consumo Máx</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Kg Mín</t>
+          <t>Mts compra Mín (+SS)</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Kg Máx</t>
+          <t>Mts compra Máx (+SS)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>Kg compra Mín</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Kg compra Máx</t>
         </is>
       </c>
     </row>
@@ -2855,17 +2888,23 @@
       <c r="D5" t="n">
         <v>388</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" t="n">
         <v>445.85</v>
       </c>
-      <c r="F5" s="24" t="n">
+      <c r="F5" t="n">
         <v>485.92</v>
       </c>
-      <c r="G5" s="23" t="n">
-        <v>47.955</v>
-      </c>
-      <c r="H5" s="24" t="n">
-        <v>52.265</v>
+      <c r="G5" s="7" t="n">
+        <v>535.02</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>583.1</v>
+      </c>
+      <c r="I5" s="23" t="n">
+        <v>57.546</v>
+      </c>
+      <c r="J5" s="24" t="n">
+        <v>62.718</v>
       </c>
     </row>
     <row r="6">
@@ -2885,17 +2924,23 @@
       <c r="D6" t="n">
         <v>291</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" t="n">
         <v>334.32</v>
       </c>
-      <c r="F6" s="24" t="n">
+      <c r="F6" t="n">
         <v>364.33</v>
       </c>
-      <c r="G6" s="23" t="n">
-        <v>35.959</v>
-      </c>
-      <c r="H6" s="24" t="n">
-        <v>39.187</v>
+      <c r="G6" s="7" t="n">
+        <v>401.18</v>
+      </c>
+      <c r="H6" s="8" t="n">
+        <v>437.2</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>43.151</v>
+      </c>
+      <c r="J6" s="24" t="n">
+        <v>47.024</v>
       </c>
     </row>
     <row r="7">
@@ -2915,17 +2960,23 @@
       <c r="D7" t="n">
         <v>291</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" t="n">
         <v>334.32</v>
       </c>
-      <c r="F7" s="24" t="n">
+      <c r="F7" t="n">
         <v>364.33</v>
       </c>
-      <c r="G7" s="23" t="n">
-        <v>35.959</v>
-      </c>
-      <c r="H7" s="24" t="n">
-        <v>39.187</v>
+      <c r="G7" s="7" t="n">
+        <v>401.18</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>437.2</v>
+      </c>
+      <c r="I7" s="23" t="n">
+        <v>43.151</v>
+      </c>
+      <c r="J7" s="24" t="n">
+        <v>47.024</v>
       </c>
     </row>
     <row r="8">
@@ -2940,17 +2991,23 @@
       <c r="D8" t="n">
         <v>970</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" t="n">
         <v>1114.49</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" t="n">
         <v>1214.58</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>119.873</v>
+        <v>1337.39</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>130.639</v>
+        <v>1457.5</v>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>143.848</v>
+      </c>
+      <c r="J8" s="10" t="n">
+        <v>156.767</v>
       </c>
     </row>
     <row r="10">
@@ -2998,12 +3055,17 @@
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Mts</t>
+          <t>Mts consumo</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Kg</t>
+          <t>Mts compra (+SS)</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Kg compra (+SS)</t>
         </is>
       </c>
     </row>
@@ -3034,8 +3096,11 @@
       <c r="H12" t="n">
         <v>485.92</v>
       </c>
-      <c r="I12" t="n">
-        <v>52.265</v>
+      <c r="I12" s="8" t="n">
+        <v>583.1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>62.718</v>
       </c>
     </row>
     <row r="13">
@@ -3065,8 +3130,11 @@
       <c r="H13" t="n">
         <v>364.33</v>
       </c>
-      <c r="I13" t="n">
-        <v>39.187</v>
+      <c r="I13" s="8" t="n">
+        <v>437.2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>47.024</v>
       </c>
     </row>
     <row r="14">
@@ -3096,8 +3164,11 @@
       <c r="H14" t="n">
         <v>364.33</v>
       </c>
-      <c r="I14" t="n">
-        <v>39.187</v>
+      <c r="I14" s="8" t="n">
+        <v>437.2</v>
+      </c>
+      <c r="J14" t="n">
+        <v>47.024</v>
       </c>
     </row>
     <row r="16">
@@ -3231,7 +3302,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:J1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4230,7 +4301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -4515,6 +4586,13 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Ajustar Colección Lite: rango 1280–1350, factor temporada ×1,4 y stock
- PROD_RANGE_MIN/MAX = 1280/1350 (Chaqueta Lite + Lite Pant)
- HIGH_SEASON_FACTOR = 1.40 (escenario diciembre)
- Resumen y metodología: SS producción +15%, SS tela +20%, stock PT en taller

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.25</v>
+        <v>1.4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>439.6</v>
+        <v>492.3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>503.7</v>
+        <v>556.4</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>── COBERTURA Y STOCK DE SEGURIDAD ──</t>
+          <t>── COBERTURA Y STOCK ──</t>
         </is>
       </c>
     </row>
@@ -838,182 +838,191 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Stock de seguridad</t>
+          <t>Stock de seguridad producción</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>+15%</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>sobre demanda teórica</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Demanda teórica mín (sin cap cierres)</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1448</v>
+          <t>Stock de seguridad tela (compra)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>+20%</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>und</t>
+          <t>sobre consumo VIORI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Demanda teórica máx (sin cap cierres)</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2027</v>
+          <t>Stock PT en taller</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Contemplado</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
+          <t>buffer operativo pre-distribución y reposición</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Demanda teórica mín (referencia)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>und</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Demanda teórica máx (referencia)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2240</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>── INSUMO LIMITANTE: CIERRES QX NEGRO 0580 ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Inventario global (60 + 75 cm)</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>1492</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>und disponibles</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · Cierres 60 cm en stock</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>748</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>und</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · Cierres 75 cm en stock</t>
+          <t>Inventario global (60 + 75 cm)</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>744</v>
+        <v>1492</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>und (adaptables a 60 cm)</t>
+          <t>und disponibles</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Lógica</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1 cierre = 1 chaqueta · pool global intercambiable</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr"/>
+          <t xml:space="preserve">  · Cierres 60 cm en stock</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>748</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Tope producción (inventario global)</t>
+          <t xml:space="preserve">  · Cierres 75 cm en stock</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1492</v>
+        <v>744</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>und</t>
+          <t>und (adaptables a 60 cm)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>¿Rango 890–970 cabe en stock?</t>
+          <t>Lógica</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>1 cierre = 1 chaqueta · pool global intercambiable</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Tope producción (inventario global)</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1492</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>¿Rango 1280–1350 cabe en stock?</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>SÍ</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>── RANGO DE PRODUCCIÓN (ACORDADO) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>MÍNIMO (compromiso)</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>890</v>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>MÁXIMO</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>970</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>und</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rango de acción</t>
+          <t>MÍNIMO (compromiso)</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>80</v>
+        <v>1280</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1024,107 +1033,111 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cierres usados al mínimo</t>
+          <t>MÁXIMO</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>890</v>
+        <v>1350</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>de 1492 disp.</t>
+          <t>und</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cierres usados al máximo</t>
+          <t>Rango de acción</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>970</v>
+        <v>70</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>de 1492 disp.</t>
+          <t>und</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>Cierres usados al mínimo</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1280</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>de 1492 disp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Cierres usados al máximo</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1350</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>de 1492 disp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>Remanente global al máximo</t>
         </is>
       </c>
-      <c r="B37" t="n">
-        <v>522</v>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B39" t="n">
+        <v>142</v>
+      </c>
+      <c r="C39" t="inlineStr">
         <is>
           <t>und</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>── COLORES DE PRODUCCIÓN ──</t>
         </is>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>Negro</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>40%</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>protagonista</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Vinotinto</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Verde Militar</t>
+          <t>Negro</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>30%</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr"/>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>protagonista</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Curva completa color × talla</t>
+          <t>Vinotinto</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Hoja Cantidades por Colores</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="C43" t="inlineStr"/>
@@ -1132,12 +1145,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Detalle color/talla Mín-Máx</t>
+          <t>Verde Militar</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Hoja Producción Color × Talla</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="C44" t="inlineStr"/>
@@ -1145,61 +1158,57 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>Curva completa color × talla</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Hoja Cantidades por Colores</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Detalle color/talla Mín-Máx</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Hoja Producción Color × Talla</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>Compra tela VIORI</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Hoja Compra de Tela (+20% SS)</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="C47" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B48" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Tolón proyectado (85% Chacao)</t>
-        </is>
-      </c>
-      <c r="B49" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Web histórica</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1210,11 +1219,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>37.2</v>
+        <v>60.4</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1225,11 +1234,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>10</v>
+        <v>7.8</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1240,11 +1249,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>77.7</v>
+        <v>37.2</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1255,11 +1264,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>8.300000000000001</v>
+        <v>10</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1270,11 +1279,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>14</v>
+        <v>77.7</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1285,11 +1294,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>Grand Plaz histórica</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>64.09999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1300,45 +1309,75 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>14</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Notas</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+          <t>Notas</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
@@ -1433,16 +1472,16 @@
         <v>60</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>216</v>
+        <v>310</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>235</v>
+        <v>327</v>
       </c>
       <c r="F5" t="n">
-        <v>216</v>
+        <v>310</v>
       </c>
       <c r="G5" t="n">
-        <v>235</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6">
@@ -1460,16 +1499,16 @@
         <v>60</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>259</v>
+        <v>373</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>283</v>
+        <v>394</v>
       </c>
       <c r="F6" t="n">
-        <v>259</v>
+        <v>373</v>
       </c>
       <c r="G6" t="n">
-        <v>283</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7">
@@ -1487,16 +1526,16 @@
         <v>60</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>247</v>
+        <v>355</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>269</v>
+        <v>374</v>
       </c>
       <c r="F7" t="n">
-        <v>247</v>
+        <v>355</v>
       </c>
       <c r="G7" t="n">
-        <v>269</v>
+        <v>374</v>
       </c>
     </row>
     <row r="8">
@@ -1514,16 +1553,16 @@
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>148</v>
+        <v>206</v>
       </c>
       <c r="F8" t="n">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="G8" t="n">
-        <v>148</v>
+        <v>206</v>
       </c>
     </row>
     <row r="9">
@@ -1541,16 +1580,16 @@
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="F9" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="G9" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10">
@@ -1560,16 +1599,16 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>722</v>
+        <v>1038</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>787</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="12">
@@ -1583,7 +1622,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Usa máx 970 (65%)</t>
+          <t>Usa máx 1350 (90%)</t>
         </is>
       </c>
     </row>
@@ -1594,11 +1633,11 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>522</v>
+        <v>142</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Incl. 39 cierres 75→60 cm</t>
+          <t>Incl. 347 cierres 75→60 cm</t>
         </is>
       </c>
     </row>
@@ -1643,14 +1682,14 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>Rango producción: 890 – 970 und</t>
+          <t>Rango producción: 1280 – 1350 und</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>MÍNIMO — 890 und (compromiso)</t>
+          <t>MÍNIMO — 1280 und (compromiso)</t>
         </is>
       </c>
     </row>
@@ -1698,22 +1737,22 @@
         </is>
       </c>
       <c r="B7" s="18" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="C7" s="18" t="n">
-        <v>104</v>
+        <v>149</v>
       </c>
       <c r="D7" s="18" t="n">
-        <v>99</v>
+        <v>142</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G7" s="18" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
     </row>
     <row r="8">
@@ -1723,22 +1762,22 @@
         </is>
       </c>
       <c r="B8" s="18" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G8" s="18" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
     </row>
     <row r="9">
@@ -1748,22 +1787,22 @@
         </is>
       </c>
       <c r="B9" s="18" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="D9" s="18" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
     </row>
     <row r="10">
@@ -1773,28 +1812,28 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>216</v>
+        <v>310</v>
       </c>
       <c r="C10" s="20" t="n">
-        <v>260</v>
+        <v>373</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>247</v>
+        <v>354</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>136</v>
+        <v>196</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="G10" s="20" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>MÁXIMO — 970 und (techo)</t>
+          <t>MÁXIMO — 1350 und (techo)</t>
         </is>
       </c>
     </row>
@@ -1842,22 +1881,22 @@
         </is>
       </c>
       <c r="B14" s="18" t="n">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>113</v>
+        <v>157</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
     </row>
     <row r="15">
@@ -1867,22 +1906,22 @@
         </is>
       </c>
       <c r="B15" s="18" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C15" s="18" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D15" s="18" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G15" s="18" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="16">
@@ -1892,22 +1931,22 @@
         </is>
       </c>
       <c r="B16" s="18" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17">
@@ -1917,22 +1956,22 @@
         </is>
       </c>
       <c r="B17" s="20" t="n">
-        <v>236</v>
+        <v>327</v>
       </c>
       <c r="C17" s="20" t="n">
-        <v>283</v>
+        <v>393</v>
       </c>
       <c r="D17" s="20" t="n">
-        <v>270</v>
+        <v>374</v>
       </c>
       <c r="E17" s="20" t="n">
-        <v>147</v>
+        <v>207</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="G17" s="20" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="19">
@@ -1976,10 +2015,10 @@
         </is>
       </c>
       <c r="B21" s="23" t="n">
-        <v>445.85</v>
+        <v>641.27</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>485.92</v>
+        <v>676.3</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1999,10 +2038,10 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>535.02</v>
+        <v>769.52</v>
       </c>
       <c r="C22" s="24" t="n">
-        <v>583.1</v>
+        <v>811.5599999999999</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2011,7 +2050,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>62.718 kg al máx</t>
+          <t>87.29 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2022,10 +2061,10 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>401.18</v>
+        <v>577.14</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>437.2</v>
+        <v>608.72</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2034,7 +2073,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>47.024 kg al máx</t>
+          <t>65.473 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2045,10 +2084,10 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>401.18</v>
+        <v>577.14</v>
       </c>
       <c r="C24" s="24" t="n">
-        <v>437.2</v>
+        <v>608.72</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2057,7 +2096,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>47.024 kg al máx</t>
+          <t>65.473 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2068,10 +2107,10 @@
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>1337.39</v>
+        <v>1923.8</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>1457.5</v>
+        <v>2029.01</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2080,7 +2119,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>156.767 kg al máx · SS 20%</t>
+          <t>218.237 kg al máx · SS 20%</t>
         </is>
       </c>
     </row>
@@ -2091,10 +2130,10 @@
         </is>
       </c>
       <c r="B26" s="23" t="n">
-        <v>440.09</v>
+        <v>632.95</v>
       </c>
       <c r="C26" s="24" t="n">
-        <v>479.65</v>
+        <v>667.5599999999999</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2114,10 +2153,10 @@
         </is>
       </c>
       <c r="B27" s="23" t="n">
-        <v>475.69</v>
+        <v>684.15</v>
       </c>
       <c r="C27" s="24" t="n">
-        <v>518.45</v>
+        <v>721.5599999999999</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2137,10 +2176,10 @@
         </is>
       </c>
       <c r="B28" s="23" t="n">
-        <v>173.09</v>
+        <v>248.95</v>
       </c>
       <c r="C28" s="24" t="n">
-        <v>188.65</v>
+        <v>262.56</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2160,10 +2199,10 @@
         </is>
       </c>
       <c r="B29" s="23" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="C29" s="24" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2172,7 +2211,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Pool global 1492 und · rem. 522 al máx</t>
+          <t>Pool global 1492 und · rem. 142 al máx</t>
         </is>
       </c>
     </row>
@@ -2183,10 +2222,10 @@
         </is>
       </c>
       <c r="B30" s="26" t="n">
-        <v>722</v>
+        <v>1038</v>
       </c>
       <c r="C30" s="26" t="n">
-        <v>787</v>
+        <v>1095</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2206,10 +2245,10 @@
         </is>
       </c>
       <c r="B31" s="26" t="n">
-        <v>168</v>
+        <v>242</v>
       </c>
       <c r="C31" s="26" t="n">
-        <v>183</v>
+        <v>255</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2273,7 +2312,7 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Rango global: 890 – 970 und</t>
+          <t>Rango global: 1280 – 1350 und</t>
         </is>
       </c>
     </row>
@@ -2375,34 +2414,34 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>86</v>
+        <v>124</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>104</v>
+        <v>149</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>113</v>
+        <v>157</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>99</v>
+        <v>142</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
@@ -2412,10 +2451,10 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
     </row>
     <row r="11">
@@ -2516,34 +2555,34 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="E14" s="8" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="G14" s="8" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15">
@@ -2553,10 +2592,10 @@
         </is>
       </c>
       <c r="B15" s="10" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="17">
@@ -2657,34 +2696,34 @@
         </is>
       </c>
       <c r="B20" s="7" t="n">
-        <v>65</v>
+        <v>93</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>78</v>
+        <v>112</v>
       </c>
       <c r="E20" s="8" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>41</v>
+        <v>59</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="21">
@@ -2694,10 +2733,10 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C21" s="10" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="23">
@@ -2707,10 +2746,10 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="C23" s="10" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="25">
@@ -2727,10 +2766,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
       <c r="C26" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
     </row>
     <row r="27">
@@ -2740,10 +2779,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C27" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
     <row r="28">
@@ -2753,10 +2792,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="C28" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>
@@ -2883,28 +2922,28 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>356</v>
+        <v>512</v>
       </c>
       <c r="D5" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
       <c r="E5" t="n">
-        <v>445.85</v>
+        <v>641.27</v>
       </c>
       <c r="F5" t="n">
-        <v>485.92</v>
+        <v>676.3</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>535.02</v>
+        <v>769.52</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>583.1</v>
+        <v>811.5599999999999</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>57.546</v>
+        <v>82.76900000000001</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>62.718</v>
+        <v>87.29000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -2919,28 +2958,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="D6" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="E6" t="n">
-        <v>334.32</v>
+        <v>480.95</v>
       </c>
       <c r="F6" t="n">
-        <v>364.33</v>
+        <v>507.27</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>401.18</v>
+        <v>577.14</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>437.2</v>
+        <v>608.72</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>43.151</v>
+        <v>62.076</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>47.024</v>
+        <v>65.473</v>
       </c>
     </row>
     <row r="7">
@@ -2955,28 +2994,28 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>267</v>
+        <v>384</v>
       </c>
       <c r="D7" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="E7" t="n">
-        <v>334.32</v>
+        <v>480.95</v>
       </c>
       <c r="F7" t="n">
-        <v>364.33</v>
+        <v>507.27</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>401.18</v>
+        <v>577.14</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>437.2</v>
+        <v>608.72</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>43.151</v>
+        <v>62.076</v>
       </c>
       <c r="J7" s="24" t="n">
-        <v>47.024</v>
+        <v>65.473</v>
       </c>
     </row>
     <row r="8">
@@ -2986,28 +3025,28 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="D8" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
       <c r="E8" t="n">
-        <v>1114.49</v>
+        <v>1603.17</v>
       </c>
       <c r="F8" t="n">
-        <v>1214.58</v>
+        <v>1690.84</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1337.39</v>
+        <v>1923.8</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>1457.5</v>
+        <v>2029.01</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>143.848</v>
+        <v>206.921</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>156.767</v>
+        <v>218.237</v>
       </c>
     </row>
     <row r="10">
@@ -3076,31 +3115,31 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>94</v>
+        <v>131</v>
       </c>
       <c r="C12" t="n">
-        <v>113</v>
+        <v>157</v>
       </c>
       <c r="D12" t="n">
-        <v>108</v>
+        <v>150</v>
       </c>
       <c r="E12" t="n">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="F12" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="G12" t="n">
-        <v>388</v>
+        <v>540</v>
       </c>
       <c r="H12" t="n">
-        <v>485.92</v>
+        <v>676.3</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>583.1</v>
+        <v>811.5599999999999</v>
       </c>
       <c r="J12" t="n">
-        <v>62.718</v>
+        <v>87.29000000000001</v>
       </c>
     </row>
     <row r="13">
@@ -3110,31 +3149,31 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C13" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D13" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E13" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="F13" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G13" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="H13" t="n">
-        <v>364.33</v>
+        <v>507.27</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>437.2</v>
+        <v>608.72</v>
       </c>
       <c r="J13" t="n">
-        <v>47.024</v>
+        <v>65.473</v>
       </c>
     </row>
     <row r="14">
@@ -3144,31 +3183,31 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>71</v>
+        <v>98</v>
       </c>
       <c r="C14" t="n">
-        <v>85</v>
+        <v>118</v>
       </c>
       <c r="D14" t="n">
-        <v>81</v>
+        <v>112</v>
       </c>
       <c r="E14" t="n">
-        <v>44</v>
+        <v>62</v>
       </c>
       <c r="F14" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G14" t="n">
-        <v>291</v>
+        <v>405</v>
       </c>
       <c r="H14" t="n">
-        <v>364.33</v>
+        <v>507.27</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>437.2</v>
+        <v>608.72</v>
       </c>
       <c r="J14" t="n">
-        <v>47.024</v>
+        <v>65.473</v>
       </c>
     </row>
     <row r="16">
@@ -3268,10 +3307,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>440.09</v>
+        <v>632.95</v>
       </c>
       <c r="C22" t="n">
-        <v>479.65</v>
+        <v>667.5599999999999</v>
       </c>
     </row>
     <row r="23">
@@ -3281,10 +3320,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>475.69</v>
+        <v>684.15</v>
       </c>
       <c r="C23" t="n">
-        <v>518.45</v>
+        <v>721.5599999999999</v>
       </c>
     </row>
     <row r="24">
@@ -3294,10 +3333,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>173.09</v>
+        <v>248.95</v>
       </c>
       <c r="C24" t="n">
-        <v>188.65</v>
+        <v>262.56</v>
       </c>
     </row>
   </sheetData>
@@ -3435,34 +3474,34 @@
         </is>
       </c>
       <c r="B5" s="23" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="C5" s="24" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="D5" s="23" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="F5" s="23" t="n">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K5" s="24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -3472,34 +3511,34 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C6" s="24" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -3509,34 +3548,34 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="C7" s="24" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F7" s="23" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I7" s="24" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -3546,34 +3585,34 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C8" s="24" t="n">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="E8" s="24" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="F8" s="23" t="n">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="J8" s="23" t="n">
         <v>5</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -3583,34 +3622,34 @@
         </is>
       </c>
       <c r="B9" s="23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C9" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E9" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F9" s="23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H9" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I9" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="J9" s="26" t="n">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>1</v>
       </c>
       <c r="K9" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -3620,34 +3659,34 @@
         </is>
       </c>
       <c r="B10" s="23" t="n">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="C10" s="24" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="E10" s="24" t="n">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="F10" s="23" t="n">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -3657,34 +3696,34 @@
         </is>
       </c>
       <c r="B11" s="23" t="n">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="F11" s="23" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="G11" s="24" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="H11" s="23" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J11" s="23" t="n">
         <v>4</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -3694,34 +3733,34 @@
         </is>
       </c>
       <c r="B12" s="23" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F12" s="23" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G12" s="24" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H12" s="23" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="I12" s="24" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K12" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -3731,34 +3770,34 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="G13" s="24" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -3768,34 +3807,34 @@
         </is>
       </c>
       <c r="B14" s="10" t="n">
-        <v>216</v>
+        <v>312</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>235</v>
+        <v>329</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>260</v>
+        <v>374</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>283</v>
+        <v>394</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>245</v>
+        <v>355</v>
       </c>
       <c r="G14" s="10" t="n">
-        <v>270</v>
+        <v>375</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>137</v>
+        <v>195</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>149</v>
+        <v>206</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
@@ -3834,10 +3873,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>154</v>
+        <v>221</v>
       </c>
       <c r="C18" t="n">
-        <v>169</v>
+        <v>233</v>
       </c>
       <c r="D18" t="n">
         <v>93.3</v>
@@ -3850,10 +3889,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>100</v>
+        <v>144</v>
       </c>
       <c r="C19" t="n">
-        <v>109</v>
+        <v>152</v>
       </c>
       <c r="D19" t="n">
         <v>61</v>
@@ -3866,10 +3905,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>102</v>
+        <v>147</v>
       </c>
       <c r="C20" t="n">
-        <v>111</v>
+        <v>155</v>
       </c>
       <c r="D20" t="n">
         <v>62.1</v>
@@ -3882,10 +3921,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>117</v>
+        <v>168</v>
       </c>
       <c r="C21" t="n">
-        <v>127</v>
+        <v>177</v>
       </c>
       <c r="D21" t="n">
         <v>71</v>
@@ -3898,10 +3937,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C22" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D22" t="n">
         <v>14</v>
@@ -3914,10 +3953,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>128</v>
+        <v>184</v>
       </c>
       <c r="C23" t="n">
-        <v>139</v>
+        <v>194</v>
       </c>
       <c r="D23" t="n">
         <v>77.7</v>
@@ -3930,10 +3969,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>99</v>
+        <v>143</v>
       </c>
       <c r="C24" t="n">
-        <v>108</v>
+        <v>151</v>
       </c>
       <c r="D24" t="n">
         <v>60.4</v>
@@ -3946,10 +3985,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="C25" t="n">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="D25" t="n">
         <v>37.2</v>
@@ -3962,10 +4001,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>106</v>
+        <v>152</v>
       </c>
       <c r="C26" t="n">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="D26" t="n">
         <v>64.09999999999999</v>
@@ -4149,10 +4188,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>722</v>
+        <v>1038</v>
       </c>
       <c r="D14" t="n">
-        <v>787</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="15">
@@ -4167,10 +4206,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>168</v>
+        <v>242</v>
       </c>
       <c r="D15" t="n">
-        <v>183</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16">
@@ -4181,16 +4220,16 @@
       </c>
       <c r="B16" t="inlineStr"/>
       <c r="C16" t="n">
-        <v>890</v>
+        <v>1280</v>
       </c>
       <c r="D16" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>── ASIGNACIÓN AL MÁXIMO (970 und) ──</t>
+          <t>── ASIGNACIÓN AL MÁXIMO (1350 und) ──</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4262,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>347</v>
       </c>
     </row>
     <row r="22">
@@ -4233,7 +4272,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>183</v>
+        <v>255</v>
       </c>
     </row>
     <row r="23">
@@ -4243,7 +4282,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>222</v>
+        <v>602</v>
       </c>
     </row>
     <row r="24">
@@ -4253,7 +4292,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>970</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="25">
@@ -4263,7 +4302,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>522</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27">
@@ -4274,7 +4313,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>890 – 970 und</t>
+          <t>1280 – 1350 und</t>
         </is>
       </c>
     </row>
@@ -4301,7 +4340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A46"/>
+  <dimension ref="A1:A52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -4358,149 +4397,149 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Factor ×1.25 (diciembre). Diciembre 2025 combinado: 685 und.</t>
+          <t xml:space="preserve">   Factor ×1.4 (diciembre — incrementado para escenario temporada alta).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr"/>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Diciembre 2025 combinado: 685 und.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>3. AJUSTES DE TIENDA (según indicación)</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Tolón: proyectado al 85% de Chacao (71 → 60 und/mes).</t>
+          <t xml:space="preserve">   STOCK DE SEGURIDAD Y TALLER</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Histórico Tolón: 8 und/mes — subestimado por tienda nueva.</t>
+          <t xml:space="preserve">   • Producción: +15% SS sobre demanda teórica.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Web: proyectada al 60% de Cerro Verde (62 → 37 und/mes).</t>
+          <t xml:space="preserve">   • Tela (compra): +20% SS sobre consumo VIORI.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Histórico Web: 8 und/mes.</t>
+          <t xml:space="preserve">   • Producto terminado en taller: buffer operativo (pre-distribución a tiendas y reposición).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • La Vela (nueva): promedio Sambil + Cerro Verde = 78 und/mes.</t>
-        </is>
-      </c>
+      <c r="A16" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Histórico La Vela: 10 und/mes.</t>
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>3. AJUSTES DE TIENDA (según indicación)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Grand Plaz: histórico × 1.68 (+68%) = 14 und/mes.</t>
+          <t xml:space="preserve">   • Tolón: proyectado al 85% de Chacao (71 → 60 und/mes).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">     Histórico Grand Plaz: 8 und/mes.</t>
+          <t xml:space="preserve">     Histórico Tolón: 8 und/mes — subestimado por tienda nueva.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Barquisimeto (nueva): promedio Grieta + Chacao + Tolón proyectado = 64 und/mes.</t>
+          <t xml:space="preserve">   • Web: proyectada al 60% de Cerro Verde (62 → 37 und/mes).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Corporativo: EXCLUIDO.</t>
+          <t xml:space="preserve">     Histórico Web: 8 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • La Vela (nueva): promedio Sambil + Cerro Verde = 78 und/mes.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
-        <is>
-          <t>4. RANGO GLOBAL ACORDADO</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Histórico La Vela: 10 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mínimo: 890 und | Máximo: 970 und.</t>
+          <t xml:space="preserve">   • Grand Plaz: histórico × 1.68 (+68%) = 14 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Demanda teórica calculada: 1448 – 2027 und (referencia).</t>
+          <t xml:space="preserve">     Histórico Grand Plaz: 8 und/mes.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr"/>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Barquisimeto (nueva): promedio Grieta + Chacao + Tolón proyectado = 64 und/mes.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
-        <is>
-          <t>5. INSUMO LIMITANTE — CIERRES (INVENTARIO GLOBAL)</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Corporativo: EXCLUIDO.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Stock total: 748 (60 cm) + 744 (75 cm) = 1492 und.</t>
-        </is>
-      </c>
+      <c r="A28" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Los cierres 75 cm se adaptan a 60 cm → se considera pool global intercambiable.</t>
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>4. RANGO GLOBAL ACORDADO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Tope producción = 1492 und (1 cierre por chaqueta).</t>
+          <t xml:space="preserve">   Mínimo: 1280 und | Máximo: 1350 und.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Al máximo (970 und) quedan 522 cierres remanentes.</t>
+          <t xml:space="preserve">   Demanda teórica calculada: 1600 – 2240 und (referencia).</t>
         </is>
       </c>
     </row>
@@ -4510,88 +4549,126 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>6. RANGO MÍNIMO / MÁXIMO</t>
+          <t>5. INSUMO LIMITANTE — CIERRES (INVENTARIO GLOBAL)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Compromiso mín: 890 und.</t>
+          <t xml:space="preserve">   Stock total: 748 (60 cm) + 744 (75 cm) = 1492 und.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Techo máx: 970 und.</t>
+          <t xml:space="preserve">   Los cierres 75 cm se adaptan a 60 cm → se considera pool global intercambiable.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr"/>
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tope producción = 1492 und (1 cierre por chaqueta).</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Al máximo (1350 und) quedan 142 cierres remanentes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>6. RANGO MÍNIMO / MÁXIMO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Compromiso mín: 1280 und.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Techo máx: 1350 und.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>7. DISTRIBUCIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
-        <is>
-          <t>8. COLORES Y COMPRA DE TELA</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>8. COLORES Y COMPRA DE TELA</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
         </is>

</xml_diff>

<commit_message>
Ajuste curva tallas: +1,5 pp XL desde L (Pant y Chaqueta)
- TALLA_SHIFT_L_TO_XL = 0.015 en ambos scripts (XS sin cambio)
- Pant: M/S fijas + shift L→XL; Chaqueta: shift L→XL sobre histórica
- Resumen y Metodología documentan el ajuste en ambos Excel
- Regenerados LITE_PANT y CHAQUETA_LITE con curva final

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
+++ b/CHAQUETA_LITE_RANGO_PRODUCCION.xlsx
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1197,78 +1197,55 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
+          <t>── AJUSTE CURVA TALLAS ──</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tolón histórico</t>
-        </is>
-      </c>
-      <c r="B50" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>und/mes</t>
-        </is>
-      </c>
+          <t>Curva histórica (Jacket 1.0 + 2.0)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Dashboards combinados</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tolón proyectado (85% Chacao)</t>
-        </is>
-      </c>
-      <c r="B51" t="n">
-        <v>60.4</v>
+          <t>XL (+1.5 pp ← L)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>XL 5.1%</t>
+        </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>und/mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Web histórica</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>7.8</v>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+          <t>hist XL 3.6% · L 13.8% · XS sin cambio</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Web proyectada (60% Cerro Verde)</t>
-        </is>
-      </c>
-      <c r="B53" t="n">
-        <v>37.2</v>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>und/mes</t>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>── AJUSTES DE TIENDA (DISTRIBUCIÓN) ──</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>La Vela histórica</t>
+          <t>Tolón histórico</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>10</v>
+        <v>8.1</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1279,11 +1256,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+          <t>Tolón proyectado (85% Chacao)</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>77.7</v>
+        <v>60.4</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1294,11 +1271,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Grand Plaz histórica</t>
+          <t>Web histórica</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>8.300000000000001</v>
+        <v>7.8</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1309,11 +1286,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Grand Plaz proyectada (+68% hist.)</t>
+          <t>Web proyectada (60% Cerro Verde)</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>14</v>
+        <v>37.2</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1324,11 +1301,11 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+          <t>La Vela histórica</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>64.09999999999999</v>
+        <v>10</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1339,45 +1316,105 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Corporativo</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>EXCLUIDO</t>
+          <t>La Vela proyectada (avg Sambil + Cerro Verde)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>und/mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Grand Plaz histórica</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Notas</t>
+          <t>Grand Plaz proyectada (+68% hist.)</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>14</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+          <t>Barquisimeto (avg Grieta+Chacao+Tolón proy.)</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>und/mes</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>• Solo género DAMA, tallas XS a XL.</t>
+          <t>Corporativo</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EXCLUIDO</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>• Dashboards adjuntos Jacket 1.0 y Jacket 2.0 leídos y combinados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>• Producto NUEVO manufacturado — sin stock inicial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>• Solo género DAMA, tallas XS a XL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>• Preferencia: 60 cm → XS/S/M · 75 cm → L/XL · excedente 75 cm adaptable a 60 cm.</t>
         </is>
@@ -1416,7 +1453,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>DAMA · Curva Jacket 1.0 + 2.0 DAMA combinado</t>
+          <t>DAMA · Curva Jacket 1.0 + 2.0 DAMA · XL +1.5 pp desde L</t>
         </is>
       </c>
     </row>
@@ -1546,23 +1583,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15.3%</t>
+          <t>13.8%</t>
         </is>
       </c>
       <c r="C8" t="n">
         <v>75</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>196</v>
+        <v>176</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>206</v>
+        <v>186</v>
       </c>
       <c r="F8" t="n">
-        <v>196</v>
+        <v>176</v>
       </c>
       <c r="G8" t="n">
-        <v>206</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9">
@@ -1573,23 +1610,23 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3.6%</t>
+          <t>5.1%</t>
         </is>
       </c>
       <c r="C9" t="n">
         <v>75</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="F9" t="n">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="G9" t="n">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10">
@@ -1746,10 +1783,10 @@
         <v>142</v>
       </c>
       <c r="E7" s="18" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G7" s="18" t="n">
         <v>512</v>
@@ -1771,10 +1808,10 @@
         <v>106</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G8" s="18" t="n">
         <v>384</v>
@@ -1796,10 +1833,10 @@
         <v>106</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G9" s="18" t="n">
         <v>384</v>
@@ -1821,10 +1858,10 @@
         <v>354</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>196</v>
+        <v>177</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="G10" s="20" t="n">
         <v>1280</v>
@@ -1890,10 +1927,10 @@
         <v>150</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G14" s="18" t="n">
         <v>540</v>
@@ -1915,10 +1952,10 @@
         <v>112</v>
       </c>
       <c r="E15" s="18" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F15" s="18" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G15" s="18" t="n">
         <v>405</v>
@@ -1940,10 +1977,10 @@
         <v>112</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G16" s="18" t="n">
         <v>405</v>
@@ -1965,10 +2002,10 @@
         <v>374</v>
       </c>
       <c r="E17" s="20" t="n">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="F17" s="20" t="n">
-        <v>49</v>
+        <v>70</v>
       </c>
       <c r="G17" s="20" t="n">
         <v>1350</v>
@@ -2015,10 +2052,10 @@
         </is>
       </c>
       <c r="B21" s="23" t="n">
-        <v>641.27</v>
+        <v>641.34</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>676.3</v>
+        <v>676.39</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2038,10 +2075,10 @@
         </is>
       </c>
       <c r="B22" s="23" t="n">
-        <v>769.52</v>
+        <v>769.61</v>
       </c>
       <c r="C22" s="24" t="n">
-        <v>811.5599999999999</v>
+        <v>811.67</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -2050,7 +2087,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>87.29 kg al máx</t>
+          <t>87.301 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2061,10 +2098,10 @@
         </is>
       </c>
       <c r="B23" s="23" t="n">
-        <v>577.14</v>
+        <v>577.21</v>
       </c>
       <c r="C23" s="24" t="n">
-        <v>608.72</v>
+        <v>608.8</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2073,7 +2110,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>65.473 kg al máx</t>
+          <t>65.48 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2084,10 +2121,10 @@
         </is>
       </c>
       <c r="B24" s="23" t="n">
-        <v>577.14</v>
+        <v>577.21</v>
       </c>
       <c r="C24" s="24" t="n">
-        <v>608.72</v>
+        <v>608.8</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -2096,7 +2133,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>65.473 kg al máx</t>
+          <t>65.48 kg al máx</t>
         </is>
       </c>
     </row>
@@ -2107,10 +2144,10 @@
         </is>
       </c>
       <c r="B25" s="23" t="n">
-        <v>1923.8</v>
+        <v>1924.03</v>
       </c>
       <c r="C25" s="24" t="n">
-        <v>2029.01</v>
+        <v>2029.26</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -2119,7 +2156,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>218.237 kg al máx · SS 20%</t>
+          <t>218.262 kg al máx · SS 20%</t>
         </is>
       </c>
     </row>
@@ -2130,10 +2167,10 @@
         </is>
       </c>
       <c r="B26" s="23" t="n">
-        <v>632.95</v>
+        <v>633.15</v>
       </c>
       <c r="C26" s="24" t="n">
-        <v>667.5599999999999</v>
+        <v>667.76</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2153,10 +2190,10 @@
         </is>
       </c>
       <c r="B27" s="23" t="n">
-        <v>684.15</v>
+        <v>684.35</v>
       </c>
       <c r="C27" s="24" t="n">
-        <v>721.5599999999999</v>
+        <v>721.76</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2176,10 +2213,10 @@
         </is>
       </c>
       <c r="B28" s="23" t="n">
-        <v>248.95</v>
+        <v>249.15</v>
       </c>
       <c r="C28" s="24" t="n">
-        <v>262.56</v>
+        <v>262.76</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2432,16 +2469,16 @@
         <v>150</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="K8" s="8" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -2573,16 +2610,16 @@
         <v>112</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="K14" s="8" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15">
@@ -2714,16 +2751,16 @@
         <v>112</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="K20" s="8" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21">
@@ -2928,22 +2965,22 @@
         <v>540</v>
       </c>
       <c r="E5" t="n">
-        <v>641.27</v>
+        <v>641.34</v>
       </c>
       <c r="F5" t="n">
-        <v>676.3</v>
+        <v>676.39</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>769.52</v>
+        <v>769.61</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>811.5599999999999</v>
+        <v>811.67</v>
       </c>
       <c r="I5" s="23" t="n">
-        <v>82.76900000000001</v>
+        <v>82.777</v>
       </c>
       <c r="J5" s="24" t="n">
-        <v>87.29000000000001</v>
+        <v>87.301</v>
       </c>
     </row>
     <row r="6">
@@ -2964,22 +3001,22 @@
         <v>405</v>
       </c>
       <c r="E6" t="n">
-        <v>480.95</v>
+        <v>481.01</v>
       </c>
       <c r="F6" t="n">
-        <v>507.27</v>
+        <v>507.33</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>577.14</v>
+        <v>577.21</v>
       </c>
       <c r="H6" s="8" t="n">
-        <v>608.72</v>
+        <v>608.8</v>
       </c>
       <c r="I6" s="23" t="n">
-        <v>62.076</v>
+        <v>62.083</v>
       </c>
       <c r="J6" s="24" t="n">
-        <v>65.473</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="7">
@@ -3000,22 +3037,22 @@
         <v>405</v>
       </c>
       <c r="E7" t="n">
-        <v>480.95</v>
+        <v>481.01</v>
       </c>
       <c r="F7" t="n">
-        <v>507.27</v>
+        <v>507.33</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>577.14</v>
+        <v>577.21</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>608.72</v>
+        <v>608.8</v>
       </c>
       <c r="I7" s="23" t="n">
-        <v>62.076</v>
+        <v>62.083</v>
       </c>
       <c r="J7" s="24" t="n">
-        <v>65.473</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="8">
@@ -3031,22 +3068,22 @@
         <v>1350</v>
       </c>
       <c r="E8" t="n">
-        <v>1603.17</v>
+        <v>1603.36</v>
       </c>
       <c r="F8" t="n">
-        <v>1690.84</v>
+        <v>1691.05</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1923.8</v>
+        <v>1924.03</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>2029.01</v>
+        <v>2029.26</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>206.921</v>
+        <v>206.944</v>
       </c>
       <c r="J8" s="10" t="n">
-        <v>218.237</v>
+        <v>218.262</v>
       </c>
     </row>
     <row r="10">
@@ -3124,22 +3161,22 @@
         <v>150</v>
       </c>
       <c r="E12" t="n">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="F12" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G12" t="n">
         <v>540</v>
       </c>
       <c r="H12" t="n">
-        <v>676.3</v>
+        <v>676.39</v>
       </c>
       <c r="I12" s="8" t="n">
-        <v>811.5599999999999</v>
+        <v>811.67</v>
       </c>
       <c r="J12" t="n">
-        <v>87.29000000000001</v>
+        <v>87.301</v>
       </c>
     </row>
     <row r="13">
@@ -3158,22 +3195,22 @@
         <v>112</v>
       </c>
       <c r="E13" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F13" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G13" t="n">
         <v>405</v>
       </c>
       <c r="H13" t="n">
-        <v>507.27</v>
+        <v>507.33</v>
       </c>
       <c r="I13" s="8" t="n">
-        <v>608.72</v>
+        <v>608.8</v>
       </c>
       <c r="J13" t="n">
-        <v>65.473</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="14">
@@ -3192,22 +3229,22 @@
         <v>112</v>
       </c>
       <c r="E14" t="n">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="F14" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G14" t="n">
         <v>405</v>
       </c>
       <c r="H14" t="n">
-        <v>507.27</v>
+        <v>507.33</v>
       </c>
       <c r="I14" s="8" t="n">
-        <v>608.72</v>
+        <v>608.8</v>
       </c>
       <c r="J14" t="n">
-        <v>65.473</v>
+        <v>65.48</v>
       </c>
     </row>
     <row r="16">
@@ -3307,10 +3344,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>632.95</v>
+        <v>633.15</v>
       </c>
       <c r="C22" t="n">
-        <v>667.5599999999999</v>
+        <v>667.76</v>
       </c>
     </row>
     <row r="23">
@@ -3320,10 +3357,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>684.15</v>
+        <v>684.35</v>
       </c>
       <c r="C23" t="n">
-        <v>721.5599999999999</v>
+        <v>721.76</v>
       </c>
     </row>
     <row r="24">
@@ -3333,10 +3370,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>248.95</v>
+        <v>249.15</v>
       </c>
       <c r="C24" t="n">
-        <v>262.56</v>
+        <v>262.76</v>
       </c>
     </row>
   </sheetData>
@@ -3492,16 +3529,16 @@
         <v>65</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="J5" s="23" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K5" s="24" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6">
@@ -3529,16 +3566,16 @@
         <v>42</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K6" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -3566,16 +3603,16 @@
         <v>43</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I7" s="24" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K7" s="24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
@@ -3603,16 +3640,16 @@
         <v>49</v>
       </c>
       <c r="H8" s="23" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="I8" s="24" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J8" s="23" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K8" s="24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -3677,16 +3714,16 @@
         <v>54</v>
       </c>
       <c r="H10" s="23" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="I10" s="24" t="n">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K10" s="24" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -3714,16 +3751,16 @@
         <v>42</v>
       </c>
       <c r="H11" s="23" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K11" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -3751,16 +3788,16 @@
         <v>26</v>
       </c>
       <c r="H12" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="I12" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="I12" s="24" t="n">
-        <v>14</v>
-      </c>
       <c r="J12" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" s="24" t="n">
         <v>4</v>
-      </c>
-      <c r="K12" s="24" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -3788,16 +3825,16 @@
         <v>44</v>
       </c>
       <c r="H13" s="23" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I13" s="24" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K13" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
@@ -3825,16 +3862,16 @@
         <v>375</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="I14" s="10" t="n">
-        <v>206</v>
+        <v>186</v>
       </c>
       <c r="J14" s="10" t="n">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="K14" s="10" t="n">
-        <v>46</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16">
@@ -4340,7 +4377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -4611,21 +4648,21 @@
     <row r="43">
       <c r="A43" s="13" t="inlineStr">
         <is>
-          <t>7. DISTRIBUCIÓN</t>
+          <t>7. AJUSTE CURVA TALLAS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
+          <t xml:space="preserve">   Histórica Jacket 1.0 + 2.0 DAMA: L 15.3% · XL 3.6%.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Por talla: curva combinada Jacket 1.0 + 2.0 DAMA.</t>
+          <t xml:space="preserve">   XL reforzado +1.5 pp desde L → L 13.8% · XL 5.1% (XS sin cambio).</t>
         </is>
       </c>
     </row>
@@ -4635,40 +4672,64 @@
     <row r="47">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>8. COLORES Y COMPRA DE TELA</t>
+          <t>8. DISTRIBUCIÓN</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
+          <t xml:space="preserve">   Por tienda: pesos mensuales proyectados (Tolón/Web/Barquisimeto ajustados).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+          <t xml:space="preserve">   Por talla: curva histórica ajustada (ver sección 7).</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
-        </is>
-      </c>
+      <c r="A50" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>9. COLORES Y COMPRA DE TELA</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Colores: Negro 40% · Vinotinto 30% · Verde Militar 30%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Dentro de cada color se aplica la misma curva de tallas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Consumo VIORI por pieza (ficha técnica): XS 1.19m · S 1.22m · M 1.28m · L 1.34m · XL 1.35m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Stock de seguridad tela: +20% sobre consumo (compra = consumo × 1.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t xml:space="preserve">   Ver hojas 'Producción Color × Talla' y 'Compra de Tela VIORI'.</t>
         </is>

</xml_diff>